<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 20:29 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -5440,7 +5440,7 @@
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="9">
-        <v>46146.94140628472</v>
+        <v>46197.83476153935</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>242</v>
@@ -5449,10 +5449,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>223</v>
+        <v>161</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>224</v>
+        <v>162</v>
       </c>
       <c r="I67" s="10"/>
       <c r="J67" s="9">
@@ -5501,7 +5501,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46146.941706412035</v>
+        <v>46197.83481741898</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>228</v>
@@ -5510,10 +5510,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>223</v>
+        <v>161</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>224</v>
+        <v>162</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="5">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="9">
-        <v>46146.94170292824</v>
+        <v>46197.83486086805</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>228</v>
@@ -5561,10 +5561,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>223</v>
+        <v>161</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>224</v>
+        <v>162</v>
       </c>
       <c r="I69" s="10"/>
       <c r="J69" s="9">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 18:15 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -3435,7 +3435,7 @@
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46197.71192840278</v>
+        <v>46198.71236186342</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>128</v>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46197.7115691088</v>
+        <v>46198.71406938657</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>180</v>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="9">
-        <v>46197.71167261574</v>
+        <v>46198.71808170139</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 13:14 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -1729,13 +1729,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46146.62019984954</v>
+        <v>46146.7868665162</v>
       </c>
       <c r="C4" s="5">
-        <v>46175.70543086805</v>
+        <v>46175.872097534724</v>
       </c>
       <c r="D4" s="5">
-        <v>46175.70544517361</v>
+        <v>46175.872111840275</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1782,13 +1782,13 @@
         <v>28</v>
       </c>
       <c r="B5" s="9">
-        <v>46146.620326226854</v>
+        <v>46146.78699289352</v>
       </c>
       <c r="C5" s="9">
-        <v>46175.70540511574</v>
+        <v>46175.8720717824</v>
       </c>
       <c r="D5" s="9">
-        <v>46175.70543134259</v>
+        <v>46175.87209800926</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>29</v>
@@ -1845,13 +1845,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46146.62032965278</v>
+        <v>46146.786996319446</v>
       </c>
       <c r="C6" s="5">
-        <v>46175.70540572917</v>
+        <v>46175.87207239583</v>
       </c>
       <c r="D6" s="5">
-        <v>46175.70543135417</v>
+        <v>46175.87209802083</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1908,13 +1908,13 @@
         <v>37</v>
       </c>
       <c r="B7" s="9">
-        <v>46146.620332997685</v>
+        <v>46146.78699966436</v>
       </c>
       <c r="C7" s="9">
-        <v>46175.705406099536</v>
+        <v>46175.8720727662</v>
       </c>
       <c r="D7" s="9">
-        <v>46175.70543190972</v>
+        <v>46175.872098576394</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>38</v>
@@ -1971,13 +1971,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46146.62033583333</v>
+        <v>46146.7870025</v>
       </c>
       <c r="C8" s="5">
-        <v>46175.705406469904</v>
+        <v>46175.872073136576</v>
       </c>
       <c r="D8" s="5">
-        <v>46175.70543217592</v>
+        <v>46175.87209884259</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -2034,13 +2034,13 @@
         <v>44</v>
       </c>
       <c r="B9" s="9">
-        <v>46146.62033996527</v>
+        <v>46146.787006631945</v>
       </c>
       <c r="C9" s="9">
-        <v>46175.705407002315</v>
+        <v>46175.87207366899</v>
       </c>
       <c r="D9" s="9">
-        <v>46175.70543275463</v>
+        <v>46175.87209942129</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>45</v>
@@ -2097,13 +2097,13 @@
         <v>47</v>
       </c>
       <c r="B10" s="5">
-        <v>46146.620205439816</v>
+        <v>46146.78687210648</v>
       </c>
       <c r="C10" s="5">
-        <v>46197.482801192135</v>
+        <v>46197.64946785879</v>
       </c>
       <c r="D10" s="5">
-        <v>46197.48281369213</v>
+        <v>46197.6494803588</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>48</v>
@@ -2150,13 +2150,13 @@
         <v>50</v>
       </c>
       <c r="B11" s="9">
-        <v>46146.62034349537</v>
+        <v>46146.787010162036</v>
       </c>
       <c r="C11" s="9">
-        <v>46197.48154974537</v>
+        <v>46197.64821641204</v>
       </c>
       <c r="D11" s="9">
-        <v>46197.481566319446</v>
+        <v>46197.64823298611</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>51</v>
@@ -2215,13 +2215,13 @@
         <v>56</v>
       </c>
       <c r="B12" s="5">
-        <v>46146.62034891204</v>
+        <v>46146.7870155787</v>
       </c>
       <c r="C12" s="5">
-        <v>46197.482300578704</v>
+        <v>46197.648967245375</v>
       </c>
       <c r="D12" s="5">
-        <v>46197.48231569445</v>
+        <v>46197.64898236111</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>57</v>
@@ -2280,13 +2280,13 @@
         <v>60</v>
       </c>
       <c r="B13" s="9">
-        <v>46146.620354733794</v>
+        <v>46146.787021400465</v>
       </c>
       <c r="C13" s="9">
-        <v>46197.48278497685</v>
+        <v>46197.64945164352</v>
       </c>
       <c r="D13" s="9">
-        <v>46197.48280087963</v>
+        <v>46197.6494675463</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>61</v>
@@ -2345,11 +2345,11 @@
         <v>64</v>
       </c>
       <c r="B14" s="5">
-        <v>46146.62020984954</v>
+        <v>46146.7868765162</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46191.61742905092</v>
+        <v>46191.784095717594</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>65</v>
@@ -2392,11 +2392,11 @@
         <v>67</v>
       </c>
       <c r="B15" s="9">
-        <v>46146.620374895836</v>
+        <v>46146.7870415625</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="9">
-        <v>46199.64401516203</v>
+        <v>46199.810681828705</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>68</v>
@@ -2455,11 +2455,11 @@
         <v>71</v>
       </c>
       <c r="B16" s="5">
-        <v>46146.62038076389</v>
+        <v>46146.78704743055</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46197.4823237963</v>
+        <v>46197.64899046296</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>72</v>
@@ -2518,13 +2518,13 @@
         <v>74</v>
       </c>
       <c r="B17" s="9">
-        <v>46146.62038653935</v>
+        <v>46146.78705320602</v>
       </c>
       <c r="C17" s="9">
-        <v>46191.61742108796</v>
+        <v>46191.784087754626</v>
       </c>
       <c r="D17" s="9">
-        <v>46197.48232390046</v>
+        <v>46197.64899056713</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>75</v>
@@ -2583,11 +2583,11 @@
         <v>78</v>
       </c>
       <c r="B18" s="5">
-        <v>46146.620392384255</v>
+        <v>46146.78705905093</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46178.00363233796</v>
+        <v>46178.17029900463</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>79</v>
@@ -2646,11 +2646,11 @@
         <v>85</v>
       </c>
       <c r="B19" s="9">
-        <v>46146.620402858796</v>
+        <v>46146.78706952547</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46178.00363422454</v>
+        <v>46178.1703008912</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>86</v>
@@ -2709,11 +2709,11 @@
         <v>88</v>
       </c>
       <c r="B20" s="5">
-        <v>46146.62040673611</v>
+        <v>46146.78707340278</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46178.00363568287</v>
+        <v>46178.170302349536</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>89</v>
@@ -2772,11 +2772,11 @@
         <v>91</v>
       </c>
       <c r="B21" s="9">
-        <v>46146.62041070602</v>
+        <v>46146.78707737269</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="9">
-        <v>46178.00363732639</v>
+        <v>46178.17030399306</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>92</v>
@@ -2835,11 +2835,11 @@
         <v>94</v>
       </c>
       <c r="B22" s="5">
-        <v>46146.62021439815</v>
+        <v>46146.786881064814</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46195.759687453705</v>
+        <v>46195.92635412037</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>95</v>
@@ -2882,11 +2882,11 @@
         <v>97</v>
       </c>
       <c r="B23" s="9">
-        <v>46146.6204152662</v>
+        <v>46146.78708193287</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="9">
-        <v>46169.69203420139</v>
+        <v>46169.858700868055</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>98</v>
@@ -2945,11 +2945,11 @@
         <v>102</v>
       </c>
       <c r="B24" s="5">
-        <v>46146.620420127314</v>
+        <v>46146.78708679398</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46169.6922908912</v>
+        <v>46169.858957557866</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>103</v>
@@ -3004,11 +3004,11 @@
         <v>106</v>
       </c>
       <c r="B25" s="9">
-        <v>46146.62042537037</v>
+        <v>46146.78709203703</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="9">
-        <v>46169.69230549769</v>
+        <v>46169.85897216435</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>107</v>
@@ -3063,13 +3063,13 @@
         <v>109</v>
       </c>
       <c r="B26" s="5">
-        <v>46146.62043092593</v>
+        <v>46146.78709759259</v>
       </c>
       <c r="C26" s="5">
-        <v>46195.759676851856</v>
+        <v>46195.92634351852</v>
       </c>
       <c r="D26" s="5">
-        <v>46195.75969194445</v>
+        <v>46195.92635861111</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>110</v>
@@ -3128,13 +3128,13 @@
         <v>112</v>
       </c>
       <c r="B27" s="9">
-        <v>46146.62043646991</v>
+        <v>46146.78710313658</v>
       </c>
       <c r="C27" s="9">
-        <v>46195.759660509255</v>
+        <v>46195.92632717593</v>
       </c>
       <c r="D27" s="9">
-        <v>46195.75966293982</v>
+        <v>46195.92632960648</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>113</v>
@@ -3189,13 +3189,13 @@
         <v>115</v>
       </c>
       <c r="B28" s="5">
-        <v>46146.62044230324</v>
+        <v>46146.787108969904</v>
       </c>
       <c r="C28" s="5">
-        <v>46191.61883501157</v>
+        <v>46191.78550167824</v>
       </c>
       <c r="D28" s="5">
-        <v>46195.75967141204</v>
+        <v>46195.9263380787</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>116</v>
@@ -3250,11 +3250,11 @@
         <v>118</v>
       </c>
       <c r="B29" s="9">
-        <v>46146.62044760417</v>
+        <v>46146.78711427083</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="9">
-        <v>46191.02002251157</v>
+        <v>46191.18668917824</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>119</v>
@@ -3313,11 +3313,11 @@
         <v>121</v>
       </c>
       <c r="B30" s="5">
-        <v>46146.62045268518</v>
+        <v>46146.78711935185</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46169.69239640047</v>
+        <v>46169.859063067124</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>122</v>
@@ -3372,11 +3372,11 @@
         <v>124</v>
       </c>
       <c r="B31" s="9">
-        <v>46146.620457997684</v>
+        <v>46146.78712466435</v>
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="9">
-        <v>46190.00207650463</v>
+        <v>46190.16874317129</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>125</v>
@@ -3431,11 +3431,11 @@
         <v>127</v>
       </c>
       <c r="B32" s="5">
-        <v>46146.62046320602</v>
+        <v>46146.78712987268</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46198.545695196764</v>
+        <v>46198.71236186342</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>128</v>
@@ -3490,11 +3490,11 @@
         <v>130</v>
       </c>
       <c r="B33" s="9">
-        <v>46146.62052135417</v>
+        <v>46146.78718802083</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="9">
-        <v>46190.01523118056</v>
+        <v>46190.18189784722</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>131</v>
@@ -3553,11 +3553,11 @@
         <v>135</v>
       </c>
       <c r="B34" s="5">
-        <v>46146.620526597224</v>
+        <v>46146.78719326389</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46182.00217861111</v>
+        <v>46182.168845277774</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>136</v>
@@ -3612,11 +3612,11 @@
         <v>138</v>
       </c>
       <c r="B35" s="9">
-        <v>46146.62053138889</v>
+        <v>46146.78719805555</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="9">
-        <v>46189.001982939815</v>
+        <v>46189.16864960648</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>139</v>
@@ -3671,11 +3671,11 @@
         <v>141</v>
       </c>
       <c r="B36" s="5">
-        <v>46146.62054903935</v>
+        <v>46146.78721570602</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46190.01523125</v>
+        <v>46190.18189791667</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>142</v>
@@ -3734,11 +3734,11 @@
         <v>144</v>
       </c>
       <c r="B37" s="9">
-        <v>46146.6205521875</v>
+        <v>46146.787218854166</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="9">
-        <v>46182.002176724534</v>
+        <v>46182.168843391206</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>87</v>
@@ -3787,11 +3787,11 @@
         <v>146</v>
       </c>
       <c r="B38" s="5">
-        <v>46146.62055623843</v>
+        <v>46146.78722290509</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46189.001974803235</v>
+        <v>46189.16864146991</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>147</v>
@@ -3840,11 +3840,11 @@
         <v>149</v>
       </c>
       <c r="B39" s="9">
-        <v>46146.620560069445</v>
+        <v>46146.78722673611</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="9">
-        <v>46169.6921353588</v>
+        <v>46169.85880202547</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>150</v>
@@ -3903,11 +3903,11 @@
         <v>154</v>
       </c>
       <c r="B40" s="5">
-        <v>46146.62056321759</v>
+        <v>46146.787229884256</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46185.00290997685</v>
+        <v>46185.169576643515</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>93</v>
@@ -3956,11 +3956,11 @@
         <v>156</v>
       </c>
       <c r="B41" s="9">
-        <v>46146.6205671412</v>
+        <v>46146.787233807874</v>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="9">
-        <v>46169.69264173611</v>
+        <v>46169.85930840278</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>157</v>
@@ -4009,11 +4009,11 @@
         <v>159</v>
       </c>
       <c r="B42" s="5">
-        <v>46146.75478928241</v>
+        <v>46146.92145594908</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46169.69266547453</v>
+        <v>46169.859332141205</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>160</v>
@@ -4060,11 +4060,11 @@
         <v>163</v>
       </c>
       <c r="B43" s="9">
-        <v>46146.62057075232</v>
+        <v>46146.78723741898</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="9">
-        <v>46190.01523150463</v>
+        <v>46190.1818981713</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>164</v>
@@ -4123,11 +4123,11 @@
         <v>166</v>
       </c>
       <c r="B44" s="5">
-        <v>46146.62057396991</v>
+        <v>46146.78724063658</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46182.00217998843</v>
+        <v>46182.16884665509</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>90</v>
@@ -4176,11 +4176,11 @@
         <v>168</v>
       </c>
       <c r="B45" s="9">
-        <v>46146.62057800926</v>
+        <v>46146.78724467593</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="9">
-        <v>46189.00197628472</v>
+        <v>46189.168642951394</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>169</v>
@@ -4229,11 +4229,11 @@
         <v>171</v>
       </c>
       <c r="B46" s="5">
-        <v>46146.620219097225</v>
+        <v>46146.78688576389</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46197.54429910879</v>
+        <v>46197.71096577546</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>172</v>
@@ -4276,13 +4276,13 @@
         <v>174</v>
       </c>
       <c r="B47" s="9">
-        <v>46146.62058282408</v>
+        <v>46146.78724949074</v>
       </c>
       <c r="C47" s="9">
-        <v>46197.54429189815</v>
+        <v>46197.710958564814</v>
       </c>
       <c r="D47" s="9">
-        <v>46197.54435372685</v>
+        <v>46197.711020393515</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>175</v>
@@ -4341,11 +4341,11 @@
         <v>179</v>
       </c>
       <c r="B48" s="5">
-        <v>46146.62058797454</v>
+        <v>46146.7872546412</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46198.54740271991</v>
+        <v>46198.71406938657</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>180</v>
@@ -4404,11 +4404,11 @@
         <v>183</v>
       </c>
       <c r="B49" s="9">
-        <v>46146.62059395833</v>
+        <v>46146.787260625</v>
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="9">
-        <v>46198.55141503472</v>
+        <v>46198.71808170139</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>82</v>
@@ -4465,11 +4465,11 @@
         <v>187</v>
       </c>
       <c r="B50" s="5">
-        <v>46146.620612175924</v>
+        <v>46146.78727884259</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46146.77304238426</v>
+        <v>46146.93970905093</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>188</v>
@@ -4526,11 +4526,11 @@
         <v>192</v>
       </c>
       <c r="B51" s="9">
-        <v>46146.620615949076</v>
+        <v>46146.78728261574</v>
       </c>
       <c r="C51" s="10"/>
       <c r="D51" s="9">
-        <v>46146.77290814815</v>
+        <v>46146.939574814816</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>193</v>
@@ -4577,11 +4577,11 @@
         <v>195</v>
       </c>
       <c r="B52" s="5">
-        <v>46146.62061986111</v>
+        <v>46146.787286527775</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46146.77290880787</v>
+        <v>46146.939575474535</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>193</v>
@@ -4628,11 +4628,11 @@
         <v>196</v>
       </c>
       <c r="B53" s="9">
-        <v>46146.62067509259</v>
+        <v>46146.787341759264</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="9">
-        <v>46200.517117152776</v>
+        <v>46200.68378381945</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>197</v>
@@ -4677,11 +4677,11 @@
         <v>199</v>
       </c>
       <c r="B54" s="5">
-        <v>46146.62067858796</v>
+        <v>46146.787345254634</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46200.51703649305</v>
+        <v>46200.683703159724</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>200</v>
@@ -4740,13 +4740,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="9">
-        <v>46146.62069221065</v>
+        <v>46146.787358877315</v>
       </c>
       <c r="C55" s="9">
-        <v>46200.51710871528</v>
+        <v>46200.68377538194</v>
       </c>
       <c r="D55" s="9">
-        <v>46200.51711047454</v>
+        <v>46200.6837771412</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>205</v>
@@ -4803,11 +4803,11 @@
         <v>208</v>
       </c>
       <c r="B56" s="5">
-        <v>46146.620683981484</v>
+        <v>46146.78735064815</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46192.00657780093</v>
+        <v>46192.17324446759</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>209</v>
@@ -4866,13 +4866,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="9">
-        <v>46146.630636851856</v>
+        <v>46146.79730351851</v>
       </c>
       <c r="C57" s="9">
-        <v>46200.5171996412</v>
+        <v>46200.68386630787</v>
       </c>
       <c r="D57" s="9">
-        <v>46200.517220497684</v>
+        <v>46200.683887164356</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>212</v>
@@ -4931,11 +4931,11 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46146.62068782408</v>
+        <v>46146.78735449074</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46192.00656401621</v>
+        <v>46192.17323068287</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4994,13 +4994,13 @@
         <v>217</v>
       </c>
       <c r="B59" s="9">
-        <v>46146.63084329861</v>
+        <v>46146.79750996528</v>
       </c>
       <c r="C59" s="9">
-        <v>46200.51729280093</v>
+        <v>46200.68395946759</v>
       </c>
       <c r="D59" s="9">
-        <v>46200.51730949074</v>
+        <v>46200.68397615741</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>216</v>
@@ -5059,13 +5059,13 @@
         <v>218</v>
       </c>
       <c r="B60" s="5">
-        <v>46146.62069773149</v>
+        <v>46146.787364398144</v>
       </c>
       <c r="C60" s="5">
-        <v>46200.51669892361</v>
+        <v>46200.683365590274</v>
       </c>
       <c r="D60" s="5">
-        <v>46200.516712592595</v>
+        <v>46200.68337925926</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>219</v>
@@ -5112,13 +5112,13 @@
         <v>221</v>
       </c>
       <c r="B61" s="9">
-        <v>46146.62070028935</v>
+        <v>46146.78736695602</v>
       </c>
       <c r="C61" s="9">
-        <v>46198.72679508102</v>
+        <v>46198.893461747684</v>
       </c>
       <c r="D61" s="9">
-        <v>46198.72695090278</v>
+        <v>46198.89361756944</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>222</v>
@@ -5177,13 +5177,13 @@
         <v>226</v>
       </c>
       <c r="B62" s="5">
-        <v>46146.62771714121</v>
+        <v>46146.79438380787</v>
       </c>
       <c r="C62" s="5">
-        <v>46198.72694634259</v>
+        <v>46198.89361300926</v>
       </c>
       <c r="D62" s="5">
-        <v>46200.51730047454</v>
+        <v>46200.6839671412</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>227</v>
@@ -5232,13 +5232,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="9">
-        <v>46146.627734525464</v>
+        <v>46146.79440119213</v>
       </c>
       <c r="C63" s="9">
-        <v>46198.727171562496</v>
+        <v>46198.89383822917</v>
       </c>
       <c r="D63" s="9">
-        <v>46200.51730125</v>
+        <v>46200.683967916666</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>227</v>
@@ -5287,13 +5287,13 @@
         <v>233</v>
       </c>
       <c r="B64" s="5">
-        <v>46146.620705127316</v>
+        <v>46146.78737179398</v>
       </c>
       <c r="C64" s="5">
-        <v>46198.727370567125</v>
+        <v>46198.8940372338</v>
       </c>
       <c r="D64" s="5">
-        <v>46198.72738408565</v>
+        <v>46198.894050752315</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>234</v>
@@ -5352,13 +5352,13 @@
         <v>237</v>
       </c>
       <c r="B65" s="9">
-        <v>46146.620708946764</v>
+        <v>46146.78737561342</v>
       </c>
       <c r="C65" s="9">
-        <v>46198.727355428244</v>
+        <v>46198.89402209491</v>
       </c>
       <c r="D65" s="9">
-        <v>46198.727357384254</v>
+        <v>46198.894024050926</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>227</v>
@@ -5407,13 +5407,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46146.6207152662</v>
+        <v>46146.78738193287</v>
       </c>
       <c r="C66" s="5">
-        <v>46198.72704020834</v>
+        <v>46198.893706874995</v>
       </c>
       <c r="D66" s="5">
-        <v>46198.727177939814</v>
+        <v>46198.893844606486</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>232</v>
@@ -5462,13 +5462,13 @@
         <v>241</v>
       </c>
       <c r="B67" s="9">
-        <v>46146.62073795139</v>
+        <v>46146.78740461805</v>
       </c>
       <c r="C67" s="9">
-        <v>46200.51667719908</v>
+        <v>46200.68334386574</v>
       </c>
       <c r="D67" s="9">
-        <v>46200.526537233796</v>
+        <v>46200.69320390046</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>242</v>
@@ -5525,13 +5525,13 @@
         <v>243</v>
       </c>
       <c r="B68" s="5">
-        <v>46146.62074189815</v>
+        <v>46146.787408564815</v>
       </c>
       <c r="C68" s="5">
-        <v>46200.52643666667</v>
+        <v>46200.69310333334</v>
       </c>
       <c r="D68" s="5">
-        <v>46200.52643932871</v>
+        <v>46200.69310599537</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>227</v>
@@ -5578,13 +5578,13 @@
         <v>245</v>
       </c>
       <c r="B69" s="9">
-        <v>46146.62074706018</v>
+        <v>46146.78741372685</v>
       </c>
       <c r="C69" s="9">
-        <v>46200.52652255787</v>
+        <v>46200.693189224534</v>
       </c>
       <c r="D69" s="9">
-        <v>46200.52652439815</v>
+        <v>46200.69319106481</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>227</v>
@@ -5631,11 +5631,11 @@
         <v>247</v>
       </c>
       <c r="B70" s="5">
-        <v>46146.62076790509</v>
+        <v>46146.78743457176</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46146.754552962964</v>
+        <v>46146.92121962963</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>197</v>
@@ -5678,11 +5678,11 @@
         <v>249</v>
       </c>
       <c r="B71" s="9">
-        <v>46146.62077079861</v>
+        <v>46146.787437465275</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46191.61885101852</v>
+        <v>46191.78551768519</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>250</v>
@@ -5739,11 +5739,11 @@
         <v>252</v>
       </c>
       <c r="B72" s="5">
-        <v>46146.62077674769</v>
+        <v>46146.78744341435</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46157.01592533565</v>
+        <v>46157.18259200231</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>253</v>
@@ -5800,11 +5800,11 @@
         <v>255</v>
       </c>
       <c r="B73" s="9">
-        <v>46146.620782303246</v>
+        <v>46146.7874489699</v>
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="9">
-        <v>46192.00659348379</v>
+        <v>46192.17326015046</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>256</v>
@@ -5861,11 +5861,11 @@
         <v>257</v>
       </c>
       <c r="B74" s="5">
-        <v>46146.62079372685</v>
+        <v>46146.78746039352</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46146.77516402778</v>
+        <v>46146.94183069444</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>258</v>
@@ -5922,11 +5922,11 @@
         <v>260</v>
       </c>
       <c r="B75" s="9">
-        <v>46146.6208378588</v>
+        <v>46146.78750452546</v>
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46197.422355937495</v>
+        <v>46197.58902260417</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>261</v>
@@ -5969,11 +5969,11 @@
         <v>263</v>
       </c>
       <c r="B76" s="5">
-        <v>46146.62084224537</v>
+        <v>46146.787508912035</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46200.526531678246</v>
+        <v>46200.6931983449</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>264</v>
@@ -6032,11 +6032,11 @@
         <v>266</v>
       </c>
       <c r="B77" s="9">
-        <v>46146.62085349537</v>
+        <v>46146.78752016203</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46200.5264460301</v>
+        <v>46200.693112696754</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>193</v>
@@ -6085,11 +6085,11 @@
         <v>268</v>
       </c>
       <c r="B78" s="5">
-        <v>46146.62085773148</v>
+        <v>46146.78752439815</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46200.52653221065</v>
+        <v>46200.693198877314</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>193</v>
@@ -6138,13 +6138,13 @@
         <v>269</v>
       </c>
       <c r="B79" s="9">
-        <v>46146.620914652776</v>
+        <v>46146.78758131944</v>
       </c>
       <c r="C79" s="9">
-        <v>46197.42234813658</v>
+        <v>46197.58901480324</v>
       </c>
       <c r="D79" s="9">
-        <v>46197.422360428245</v>
+        <v>46197.5890270949</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>270</v>
@@ -6201,13 +6201,13 @@
         <v>271</v>
       </c>
       <c r="B80" s="5">
-        <v>46146.62091990741</v>
+        <v>46146.78758657408</v>
       </c>
       <c r="C80" s="5">
-        <v>46197.422267581016</v>
+        <v>46197.58893424769</v>
       </c>
       <c r="D80" s="5">
-        <v>46197.42226924769</v>
+        <v>46197.58893591435</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>193</v>
@@ -6254,13 +6254,13 @@
         <v>274</v>
       </c>
       <c r="B81" s="9">
-        <v>46146.62092627315</v>
+        <v>46146.787592939814</v>
       </c>
       <c r="C81" s="9">
-        <v>46197.42233475695</v>
+        <v>46197.58900142361</v>
       </c>
       <c r="D81" s="9">
-        <v>46197.42233612269</v>
+        <v>46197.58900278935</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>193</v>
@@ -6307,11 +6307,11 @@
         <v>276</v>
       </c>
       <c r="B82" s="5">
-        <v>46146.6209508912</v>
+        <v>46146.78761755787</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46146.77531712963</v>
+        <v>46146.94198379629</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>277</v>
@@ -6370,11 +6370,11 @@
         <v>278</v>
       </c>
       <c r="B83" s="9">
-        <v>46146.620960416665</v>
+        <v>46146.78762708334</v>
       </c>
       <c r="C83" s="10"/>
       <c r="D83" s="9">
-        <v>46197.42227296296</v>
+        <v>46197.588939629626</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>193</v>
@@ -6421,11 +6421,11 @@
         <v>280</v>
       </c>
       <c r="B84" s="5">
-        <v>46146.62096664352</v>
+        <v>46146.78763331019</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46197.42234427083</v>
+        <v>46197.5890109375</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>193</v>
@@ -6472,11 +6472,11 @@
         <v>281</v>
       </c>
       <c r="B85" s="9">
-        <v>46146.62103199074</v>
+        <v>46146.78769865741</v>
       </c>
       <c r="C85" s="10"/>
       <c r="D85" s="9">
-        <v>46146.77531423611</v>
+        <v>46146.941980902775</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>282</v>
@@ -6533,11 +6533,11 @@
         <v>283</v>
       </c>
       <c r="B86" s="5">
-        <v>46146.62103688657</v>
+        <v>46146.787703553244</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46146.77562837963</v>
+        <v>46146.9422950463</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>193</v>
@@ -6584,11 +6584,11 @@
         <v>286</v>
       </c>
       <c r="B87" s="9">
-        <v>46146.62104225694</v>
+        <v>46146.78770892361</v>
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46146.7756253125</v>
+        <v>46146.94229197917</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>193</v>
@@ -6635,11 +6635,11 @@
         <v>288</v>
       </c>
       <c r="B88" s="5">
-        <v>46146.62106385417</v>
+        <v>46146.78773052084</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46146.77531146991</v>
+        <v>46146.94197813657</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>289</v>
@@ -6696,11 +6696,11 @@
         <v>290</v>
       </c>
       <c r="B89" s="9">
-        <v>46146.62106844907</v>
+        <v>46146.78773511574</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="9">
-        <v>46146.7757059375</v>
+        <v>46146.94237260417</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>193</v>
@@ -6747,11 +6747,11 @@
         <v>292</v>
       </c>
       <c r="B90" s="5">
-        <v>46146.621073692135</v>
+        <v>46146.78774035879</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46146.77570342593</v>
+        <v>46146.94237009259</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>193</v>
@@ -6798,11 +6798,11 @@
         <v>293</v>
       </c>
       <c r="B91" s="9">
-        <v>46146.6210928125</v>
+        <v>46146.787759479164</v>
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46146.77530659722</v>
+        <v>46146.94197326389</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>294</v>
@@ -6859,11 +6859,11 @@
         <v>296</v>
       </c>
       <c r="B92" s="5">
-        <v>46146.62109759259</v>
+        <v>46146.78776425926</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46146.77578200231</v>
+        <v>46146.94244866898</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>193</v>
@@ -6910,11 +6910,11 @@
         <v>298</v>
       </c>
       <c r="B93" s="9">
-        <v>46146.62110192129</v>
+        <v>46146.787768587965</v>
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46146.775778923606</v>
+        <v>46146.94244559028</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>193</v>
@@ -6961,11 +6961,11 @@
         <v>299</v>
       </c>
       <c r="B94" s="5">
-        <v>46146.62111905093</v>
+        <v>46146.78778571759</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46146.77389681713</v>
+        <v>46146.9405634838</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>300</v>
@@ -7008,11 +7008,11 @@
         <v>302</v>
       </c>
       <c r="B95" s="9">
-        <v>46146.621122453704</v>
+        <v>46146.78778912037</v>
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46146.77631427083</v>
+        <v>46146.9429809375</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>303</v>
@@ -7069,11 +7069,11 @@
         <v>307</v>
       </c>
       <c r="B96" s="5">
-        <v>46146.62112762731</v>
+        <v>46146.78779429398</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46146.77597652777</v>
+        <v>46146.942643194445</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>193</v>
@@ -7120,11 +7120,11 @@
         <v>309</v>
       </c>
       <c r="B97" s="9">
-        <v>46146.621131747685</v>
+        <v>46146.787798414356</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46146.77597726852</v>
+        <v>46146.94264393518</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>193</v>
@@ -7171,11 +7171,11 @@
         <v>311</v>
       </c>
       <c r="B98" s="5">
-        <v>46146.6211480787</v>
+        <v>46146.787814745374</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46146.77622869213</v>
+        <v>46146.94289535879</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>312</v>
@@ -7232,11 +7232,11 @@
         <v>313</v>
       </c>
       <c r="B99" s="9">
-        <v>46146.62115233796</v>
+        <v>46146.78781900463</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46146.77619097222</v>
+        <v>46146.94285763889</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>193</v>
@@ -7283,11 +7283,11 @@
         <v>315</v>
       </c>
       <c r="B100" s="5">
-        <v>46146.62115648148</v>
+        <v>46146.787823148145</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46146.77618863426</v>
+        <v>46146.94285530093</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>193</v>
@@ -7334,11 +7334,11 @@
         <v>317</v>
       </c>
       <c r="B101" s="9">
-        <v>46146.62122486111</v>
+        <v>46146.787891527776</v>
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46146.776493067126</v>
+        <v>46146.9431597338</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>318</v>
@@ -7395,11 +7395,11 @@
         <v>319</v>
       </c>
       <c r="B102" s="5">
-        <v>46146.62123096065</v>
+        <v>46146.78789762731</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46146.77676126157</v>
+        <v>46146.94342792824</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>193</v>
@@ -7446,11 +7446,11 @@
         <v>321</v>
       </c>
       <c r="B103" s="9">
-        <v>46146.62123871528</v>
+        <v>46146.78790538195</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46146.77679804398</v>
+        <v>46146.94346471065</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>193</v>
@@ -7497,11 +7497,11 @@
         <v>323</v>
       </c>
       <c r="B104" s="5">
-        <v>46146.621261504624</v>
+        <v>46146.787928171296</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46146.77660861111</v>
+        <v>46146.94327527778</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>324</v>
@@ -7558,11 +7558,11 @@
         <v>326</v>
       </c>
       <c r="B105" s="9">
-        <v>46146.62126774306</v>
+        <v>46146.787934409724</v>
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="9">
-        <v>46146.77665572916</v>
+        <v>46146.94332239583</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>193</v>
@@ -7609,11 +7609,11 @@
         <v>327</v>
       </c>
       <c r="B106" s="5">
-        <v>46146.62127246527</v>
+        <v>46146.787939131944</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46146.77665320602</v>
+        <v>46146.943319872684</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>193</v>
@@ -7660,11 +7660,11 @@
         <v>328</v>
       </c>
       <c r="B107" s="9">
-        <v>46146.62129130787</v>
+        <v>46146.787957974535</v>
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="9">
-        <v>46146.77389685185</v>
+        <v>46146.94056351852</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>329</v>
@@ -7707,11 +7707,11 @@
         <v>331</v>
       </c>
       <c r="B108" s="5">
-        <v>46146.62129487269</v>
+        <v>46146.78796153935</v>
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46146.77686291667</v>
+        <v>46146.94352958333</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>332</v>
@@ -7770,11 +7770,11 @@
         <v>335</v>
       </c>
       <c r="B109" s="9">
-        <v>46146.6213005787</v>
+        <v>46146.78796724537</v>
       </c>
       <c r="C109" s="10"/>
       <c r="D109" s="9">
-        <v>46196.701034618054</v>
+        <v>46196.86770128472</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>336</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 17:33 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="337">
   <si>
     <t>50001543 - ZITRON COLOMBIA EGM</t>
   </si>
@@ -304,30 +304,30 @@
     <t>Generación OC motor OT 4309,Propuesta compras:</t>
   </si>
   <si>
+    <t>1214511142378696</t>
+  </si>
+  <si>
+    <t>propuesta alabes OT 4309</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Alabe OT 4309</t>
+  </si>
+  <si>
+    <t>1214511142378716</t>
+  </si>
+  <si>
+    <t>propuesta nucleo rodete OT 4309</t>
+  </si>
+  <si>
+    <t>benjamin.bustos@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete OT 4309</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
   </si>
   <si>
-    <t>1214511142378696</t>
-  </si>
-  <si>
-    <t>propuesta alabes OT 4309</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Alabe OT 4309</t>
-  </si>
-  <si>
-    <t>1214511142378716</t>
-  </si>
-  <si>
-    <t>propuesta nucleo rodete OT 4309</t>
-  </si>
-  <si>
-    <t>benjamin.bustos@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete OT 4309</t>
-  </si>
-  <si>
     <t>1214511155793305</t>
   </si>
   <si>
@@ -346,58 +346,58 @@
     <t>Propuesta compras:,Generación OC materiales corte Laser OT 4309</t>
   </si>
   <si>
+    <t>1214511198886127</t>
+  </si>
+  <si>
+    <t>Propuesta Corte plasma  OT 4309</t>
+  </si>
+  <si>
+    <t>Generación OC Corte Plasma  OT 4309</t>
+  </si>
+  <si>
+    <t>1214511198886137</t>
+  </si>
+  <si>
+    <t>Propuesta Mecanizado OT 4309</t>
+  </si>
+  <si>
+    <t>Generación OC Mecanizado OT 4309</t>
+  </si>
+  <si>
+    <t>1214511198886147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta Fabricación externa OT 4309 </t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación Externa OT 4309</t>
+  </si>
+  <si>
+    <t>1214508463084762</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rodete OT 4309,Motor OT 4309,Materiales corte Laser OT 4309,Alabe OT 4309 </t>
+  </si>
+  <si>
+    <t>1214511244996574</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alabe OT 4309 </t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4309,Generación OC Alabe OT 4309</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214511198886127</t>
-  </si>
-  <si>
-    <t>Propuesta Corte plasma  OT 4309</t>
-  </si>
-  <si>
-    <t>Generación OC Corte Plasma  OT 4309</t>
-  </si>
-  <si>
-    <t>1214511198886137</t>
-  </si>
-  <si>
-    <t>Propuesta Mecanizado OT 4309</t>
-  </si>
-  <si>
-    <t>Generación OC Mecanizado OT 4309</t>
-  </si>
-  <si>
-    <t>1214511198886147</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta Fabricación externa OT 4309 </t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación Externa OT 4309</t>
-  </si>
-  <si>
-    <t>1214508463084762</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rodete OT 4309,Motor OT 4309,Materiales corte Laser OT 4309,Alabe OT 4309 </t>
-  </si>
-  <si>
-    <t>1214511244996574</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alabe OT 4309 </t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4309,Generación OC Alabe OT 4309</t>
   </si>
   <si>
     <t>1214511244996589</t>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46191.784095717594</v>
+        <v>46203.709446678244</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>65</v>
@@ -2394,9 +2394,11 @@
       <c r="B15" s="9">
         <v>46146.7870415625</v>
       </c>
-      <c r="C15" s="10"/>
+      <c r="C15" s="9">
+        <v>46203.70939159722</v>
+      </c>
       <c r="D15" s="9">
-        <v>46199.810681828705</v>
+        <v>46203.70941623843</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>68</v>
@@ -2444,25 +2446,27 @@
         <v>33</v>
       </c>
       <c r="T15" s="10">
-        <v>0</v>
-      </c>
-      <c r="U15" s="12" t="s">
-        <v>70</v>
+        <v>1</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B16" s="5">
         <v>46146.78704743055</v>
       </c>
-      <c r="C16" s="6"/>
+      <c r="C16" s="5">
+        <v>46203.70944197917</v>
+      </c>
       <c r="D16" s="5">
-        <v>46197.64899046296</v>
+        <v>46203.70945753472</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2495,7 +2499,7 @@
         <v>57</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q16" s="5">
         <v>46149</v>
@@ -2507,15 +2511,15 @@
         <v>33</v>
       </c>
       <c r="T16" s="6">
-        <v>0</v>
-      </c>
-      <c r="U16" s="12" t="s">
-        <v>70</v>
+        <v>1</v>
+      </c>
+      <c r="U16" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B17" s="9">
         <v>46146.78705320602</v>
@@ -2527,16 +2531,16 @@
         <v>46197.64899056713</v>
       </c>
       <c r="E17" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>76</v>
-      </c>
       <c r="H17" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I17" s="9">
         <v>46149</v>
@@ -2560,7 +2564,7 @@
         <v>57</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q17" s="9">
         <v>46149</v>
@@ -2575,7 +2579,7 @@
         <v>1</v>
       </c>
       <c r="U17" s="12" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
@@ -2587,7 +2591,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46178.17029900463</v>
+        <v>46203.714959756944</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>79</v>
@@ -2637,23 +2641,23 @@
       <c r="T18" s="6">
         <v>0</v>
       </c>
-      <c r="U18" s="11" t="s">
-        <v>84</v>
+      <c r="U18" s="12" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B19" s="9">
         <v>46146.78706952547</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46178.1703008912</v>
+        <v>46203.71496125</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
@@ -2686,7 +2690,7 @@
         <v>82</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Q19" s="9">
         <v>46177</v>
@@ -2700,23 +2704,23 @@
       <c r="T19" s="10">
         <v>0</v>
       </c>
-      <c r="U19" s="11" t="s">
-        <v>84</v>
+      <c r="U19" s="12" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B20" s="5">
         <v>46146.78707340278</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46178.170302349536</v>
+        <v>46203.71495998843</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2749,7 +2753,7 @@
         <v>82</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q20" s="5">
         <v>46177</v>
@@ -2763,23 +2767,23 @@
       <c r="T20" s="6">
         <v>0</v>
       </c>
-      <c r="U20" s="11" t="s">
-        <v>84</v>
+      <c r="U20" s="12" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B21" s="9">
         <v>46146.78707737269</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="9">
-        <v>46178.17030399306</v>
+        <v>46203.71496114583</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>26</v>
@@ -2812,7 +2816,7 @@
         <v>82</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q21" s="9">
         <v>46177</v>
@@ -2826,23 +2830,23 @@
       <c r="T21" s="10">
         <v>0</v>
       </c>
-      <c r="U21" s="11" t="s">
-        <v>84</v>
+      <c r="U21" s="12" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B22" s="5">
         <v>46146.786881064814</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46195.92635412037</v>
+        <v>46203.710007118054</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>25</v>
@@ -2866,7 +2870,7 @@
         <v>26</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P22" s="6" t="s">
         <v>26</v>
@@ -2879,7 +2883,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B23" s="9">
         <v>46146.78708193287</v>
@@ -2889,16 +2893,16 @@
         <v>46169.858700868055</v>
       </c>
       <c r="E23" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="10" t="s">
+      <c r="H23" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>100</v>
       </c>
       <c r="I23" s="9">
         <v>46153</v>
@@ -2916,13 +2920,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q23" s="9">
         <v>46153</v>
@@ -2937,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="U23" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -2949,7 +2953,7 @@
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46169.858957557866</v>
+        <v>46203.70944847222</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>103</v>
@@ -2958,10 +2962,10 @@
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="I24" s="5">
         <v>46153</v>
@@ -2979,10 +2983,10 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P24" s="6" t="s">
         <v>104</v>
@@ -2996,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -3017,10 +3021,10 @@
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>100</v>
       </c>
       <c r="I25" s="9">
         <v>46155</v>
@@ -3038,7 +3042,7 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O25" s="10" t="s">
         <v>103</v>
@@ -3055,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -3078,10 +3082,10 @@
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="I26" s="5">
         <v>46153</v>
@@ -3099,13 +3103,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>111</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q26" s="5">
         <v>46153</v>
@@ -3143,10 +3147,10 @@
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>100</v>
       </c>
       <c r="I27" s="9">
         <v>46153</v>
@@ -3167,7 +3171,7 @@
         <v>110</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P27" s="10" t="s">
         <v>114</v>
@@ -3181,7 +3185,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3204,10 +3208,10 @@
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="I28" s="5">
         <v>46155</v>
@@ -3242,7 +3246,7 @@
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3252,9 +3256,11 @@
       <c r="B29" s="9">
         <v>46146.78711427083</v>
       </c>
-      <c r="C29" s="10"/>
+      <c r="C29" s="9">
+        <v>46203.70999099537</v>
+      </c>
       <c r="D29" s="9">
-        <v>46191.18668917824</v>
+        <v>46203.71001635416</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>119</v>
@@ -3263,10 +3269,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>100</v>
       </c>
       <c r="I29" s="9">
         <v>46153</v>
@@ -3284,13 +3290,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O29" s="10" t="s">
         <v>120</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q29" s="9">
         <v>46153</v>
@@ -3302,10 +3308,10 @@
         <v>33</v>
       </c>
       <c r="T29" s="10">
-        <v>0</v>
-      </c>
-      <c r="U29" s="11" t="s">
-        <v>84</v>
+        <v>1</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3315,9 +3321,11 @@
       <c r="B30" s="5">
         <v>46146.78711935185</v>
       </c>
-      <c r="C30" s="6"/>
+      <c r="C30" s="5">
+        <v>46203.7099115625</v>
+      </c>
       <c r="D30" s="5">
-        <v>46169.859063067124</v>
+        <v>46203.70991413195</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>122</v>
@@ -3326,10 +3334,10 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="I30" s="5">
         <v>46153</v>
@@ -3364,7 +3372,7 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3374,9 +3382,11 @@
       <c r="B31" s="9">
         <v>46146.78712466435</v>
       </c>
-      <c r="C31" s="10"/>
+      <c r="C31" s="9">
+        <v>46203.70997548611</v>
+      </c>
       <c r="D31" s="9">
-        <v>46190.16874317129</v>
+        <v>46203.70997798612</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>125</v>
@@ -3385,10 +3395,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>100</v>
       </c>
       <c r="I31" s="9">
         <v>46162</v>
@@ -3423,7 +3433,7 @@
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3433,9 +3443,11 @@
       <c r="B32" s="5">
         <v>46146.78712987268</v>
       </c>
-      <c r="C32" s="6"/>
+      <c r="C32" s="5">
+        <v>46203.70995884259</v>
+      </c>
       <c r="D32" s="5">
-        <v>46198.71236186342</v>
+        <v>46203.709962685185</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>128</v>
@@ -3444,10 +3456,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="I32" s="5">
         <v>46161</v>
@@ -3482,7 +3494,7 @@
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -3524,13 +3536,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O33" s="10" t="s">
         <v>134</v>
       </c>
       <c r="P33" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q33" s="9">
         <v>46150</v>
@@ -3545,7 +3557,7 @@
         <v>0</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -3604,7 +3616,7 @@
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -3663,7 +3675,7 @@
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -3705,7 +3717,7 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O36" s="6" t="s">
         <v>143</v>
@@ -3726,7 +3738,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -3741,7 +3753,7 @@
         <v>46182.168843391206</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>26</v>
@@ -3771,7 +3783,7 @@
         <v>142</v>
       </c>
       <c r="O37" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="P37" s="10" t="s">
         <v>145</v>
@@ -3824,7 +3836,7 @@
         <v>142</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>148</v>
@@ -3874,7 +3886,7 @@
         <v>26</v>
       </c>
       <c r="N39" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O39" s="10" t="s">
         <v>153</v>
@@ -3895,7 +3907,7 @@
         <v>0</v>
       </c>
       <c r="U39" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -3910,7 +3922,7 @@
         <v>46185.169576643515</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
@@ -3940,7 +3952,7 @@
         <v>150</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>155</v>
@@ -3993,7 +4005,7 @@
         <v>150</v>
       </c>
       <c r="O41" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P41" s="10" t="s">
         <v>158</v>
@@ -4094,7 +4106,7 @@
         <v>26</v>
       </c>
       <c r="N43" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O43" s="10" t="s">
         <v>165</v>
@@ -4115,7 +4127,7 @@
         <v>0</v>
       </c>
       <c r="U43" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -4130,7 +4142,7 @@
         <v>46182.16884665509</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
@@ -4160,7 +4172,7 @@
         <v>164</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>167</v>
@@ -4213,7 +4225,7 @@
         <v>164</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P45" s="10" t="s">
         <v>170</v>
@@ -4233,7 +4245,7 @@
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46197.71096577546</v>
+        <v>46203.71489604167</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>172</v>
@@ -4269,7 +4281,9 @@
       <c r="R46" s="6"/>
       <c r="S46" s="6"/>
       <c r="T46" s="6"/>
-      <c r="U46" s="6"/>
+      <c r="U46" s="12" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
@@ -4343,9 +4357,11 @@
       <c r="B48" s="5">
         <v>46146.7872546412</v>
       </c>
-      <c r="C48" s="6"/>
+      <c r="C48" s="5">
+        <v>46203.714861863424</v>
+      </c>
       <c r="D48" s="5">
-        <v>46198.71406938657</v>
+        <v>46203.71488673611</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>180</v>
@@ -4393,10 +4409,10 @@
         <v>33</v>
       </c>
       <c r="T48" s="6">
-        <v>0</v>
-      </c>
-      <c r="U48" s="11" t="s">
-        <v>84</v>
+        <v>1</v>
+      </c>
+      <c r="U48" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -4406,9 +4422,11 @@
       <c r="B49" s="9">
         <v>46146.787260625</v>
       </c>
-      <c r="C49" s="10"/>
+      <c r="C49" s="9">
+        <v>46203.71491821759</v>
+      </c>
       <c r="D49" s="9">
-        <v>46198.71808170139</v>
+        <v>46203.71493509259</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>82</v>
@@ -4454,10 +4472,10 @@
         <v>33</v>
       </c>
       <c r="T49" s="10">
-        <v>0</v>
-      </c>
-      <c r="U49" s="11" t="s">
-        <v>84</v>
+        <v>1</v>
+      </c>
+      <c r="U49" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -4518,7 +4536,7 @@
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4669,7 +4687,7 @@
       <c r="S53" s="10"/>
       <c r="T53" s="10"/>
       <c r="U53" s="12" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4858,7 +4876,7 @@
         <v>0</v>
       </c>
       <c r="U56" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4986,7 +5004,7 @@
         <v>0</v>
       </c>
       <c r="U58" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -5358,7 +5376,7 @@
         <v>46198.89402209491</v>
       </c>
       <c r="D65" s="9">
-        <v>46198.894024050926</v>
+        <v>46203.71492597222</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>227</v>
@@ -5413,7 +5431,7 @@
         <v>46198.893706874995</v>
       </c>
       <c r="D66" s="5">
-        <v>46198.893844606486</v>
+        <v>46203.714927361114</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>232</v>
@@ -5517,7 +5535,7 @@
         <v>1</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5531,7 +5549,7 @@
         <v>46200.69310333334</v>
       </c>
       <c r="D68" s="5">
-        <v>46200.69310599537</v>
+        <v>46203.7149283912</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>227</v>
@@ -5584,7 +5602,7 @@
         <v>46200.693189224534</v>
       </c>
       <c r="D69" s="9">
-        <v>46200.69319106481</v>
+        <v>46203.714929317124</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>227</v>
@@ -5731,7 +5749,7 @@
         <v>0</v>
       </c>
       <c r="U71" s="12" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5792,7 +5810,7 @@
         <v>0</v>
       </c>
       <c r="U72" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5804,7 +5822,7 @@
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="9">
-        <v>46192.17326015046</v>
+        <v>46203.70999737269</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>256</v>
@@ -5852,8 +5870,8 @@
       <c r="T73" s="10">
         <v>0</v>
       </c>
-      <c r="U73" s="11" t="s">
-        <v>84</v>
+      <c r="U73" s="12" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5914,7 +5932,7 @@
         <v>0</v>
       </c>
       <c r="U74" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5982,10 +6000,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I76" s="5">
         <v>46219</v>
@@ -6024,7 +6042,7 @@
         <v>0</v>
       </c>
       <c r="U76" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6045,10 +6063,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I77" s="9">
         <v>46219</v>
@@ -6098,10 +6116,10 @@
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I78" s="5">
         <v>46219</v>
@@ -6153,10 +6171,10 @@
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H79" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="9">
@@ -6207,7 +6225,7 @@
         <v>46197.58893424769</v>
       </c>
       <c r="D80" s="5">
-        <v>46197.58893591435</v>
+        <v>46203.71494715278</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>193</v>
@@ -6216,10 +6234,10 @@
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I80" s="6"/>
       <c r="J80" s="5">
@@ -6260,7 +6278,7 @@
         <v>46197.58900142361</v>
       </c>
       <c r="D81" s="9">
-        <v>46197.58900278935</v>
+        <v>46203.71494597222</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>193</v>
@@ -6269,10 +6287,10 @@
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I81" s="10"/>
       <c r="J81" s="9">
@@ -6320,10 +6338,10 @@
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I82" s="5">
         <v>46227</v>
@@ -6362,7 +6380,7 @@
         <v>0</v>
       </c>
       <c r="U82" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6374,7 +6392,7 @@
       </c>
       <c r="C83" s="10"/>
       <c r="D83" s="9">
-        <v>46197.588939629626</v>
+        <v>46203.71494815972</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>193</v>
@@ -6383,10 +6401,10 @@
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I83" s="10"/>
       <c r="J83" s="9">
@@ -6425,7 +6443,7 @@
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46197.5890109375</v>
+        <v>46203.71494907407</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>193</v>
@@ -6434,10 +6452,10 @@
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I84" s="6"/>
       <c r="J84" s="5">
@@ -6485,10 +6503,10 @@
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I85" s="10"/>
       <c r="J85" s="9">
@@ -6525,7 +6543,7 @@
         <v>0</v>
       </c>
       <c r="U85" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -6537,7 +6555,7 @@
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46146.9422950463</v>
+        <v>46203.71494643518</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>193</v>
@@ -6546,10 +6564,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I86" s="6"/>
       <c r="J86" s="5">
@@ -6588,7 +6606,7 @@
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46146.94229197917</v>
+        <v>46203.7149375</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>193</v>
@@ -6597,10 +6615,10 @@
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I87" s="10"/>
       <c r="J87" s="9">
@@ -6648,10 +6666,10 @@
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="5">
@@ -6688,7 +6706,7 @@
         <v>0</v>
       </c>
       <c r="U88" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -6709,10 +6727,10 @@
         <v>26</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="9">
@@ -6760,10 +6778,10 @@
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="5">
@@ -6811,10 +6829,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H91" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" s="9">
@@ -6851,7 +6869,7 @@
         <v>0</v>
       </c>
       <c r="U91" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
@@ -6872,10 +6890,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I92" s="6"/>
       <c r="J92" s="5">
@@ -6923,10 +6941,10 @@
         <v>26</v>
       </c>
       <c r="G93" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H93" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="9">
@@ -7061,7 +7079,7 @@
         <v>0</v>
       </c>
       <c r="U95" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
@@ -7184,10 +7202,10 @@
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I98" s="6"/>
       <c r="J98" s="5">
@@ -7224,7 +7242,7 @@
         <v>0</v>
       </c>
       <c r="U98" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -7245,10 +7263,10 @@
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H99" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I99" s="10"/>
       <c r="J99" s="9">
@@ -7296,10 +7314,10 @@
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I100" s="6"/>
       <c r="J100" s="5">
@@ -7387,7 +7405,7 @@
         <v>0</v>
       </c>
       <c r="U101" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
@@ -7550,7 +7568,7 @@
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7762,7 +7780,7 @@
         <v>0</v>
       </c>
       <c r="U108" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
@@ -7825,7 +7843,7 @@
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-09 16:04 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1304" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="337">
   <si>
     <t>50001543 - ZITRON COLOMBIA EGM</t>
   </si>
@@ -379,6 +379,9 @@
     <t xml:space="preserve">rodete OT 4309,Motor OT 4309,Materiales corte Laser OT 4309,Alabe OT 4309 </t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1214511244996574</t>
   </si>
   <si>
@@ -394,21 +397,21 @@
     <t>Fabricación Alabe OT 4309,Generación OC Alabe OT 4309</t>
   </si>
   <si>
+    <t>1214511244996589</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4309</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Alabe OT 4309,Alabe OT 4309 </t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
   </si>
   <si>
-    <t>1214511244996589</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4309</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Alabe OT 4309,Alabe OT 4309 </t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
     <t>1214511142420461</t>
   </si>
   <si>
@@ -689,9 +692,6 @@
   </si>
   <si>
     <t xml:space="preserve">Recepcion materiales corte laser,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214511155796723</t>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46205.606627430556</v>
+        <v>46212.66398305555</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>93</v>
@@ -2893,30 +2893,34 @@
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
       <c r="T22" s="6"/>
-      <c r="U22" s="6"/>
+      <c r="U22" s="12" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B23" s="9">
         <v>46146.78708193287</v>
       </c>
-      <c r="C23" s="10"/>
+      <c r="C23" s="9">
+        <v>46212.6639628125</v>
+      </c>
       <c r="D23" s="9">
-        <v>46169.858700868055</v>
+        <v>46212.66397574074</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I23" s="9">
         <v>46153</v>
@@ -2937,7 +2941,7 @@
         <v>93</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P23" s="10" t="s">
         <v>93</v>
@@ -2952,10 +2956,10 @@
         <v>33</v>
       </c>
       <c r="T23" s="10">
-        <v>0</v>
-      </c>
-      <c r="U23" s="11" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -2965,9 +2969,11 @@
       <c r="B24" s="5">
         <v>46146.78708679398</v>
       </c>
-      <c r="C24" s="6"/>
+      <c r="C24" s="5">
+        <v>46212.66391207176</v>
+      </c>
       <c r="D24" s="5">
-        <v>46203.70944847222</v>
+        <v>46212.663913888886</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>102</v>
@@ -2976,10 +2982,10 @@
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I24" s="5">
         <v>46153</v>
@@ -2997,7 +3003,7 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>71</v>
@@ -3014,31 +3020,33 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B25" s="9">
         <v>46146.78709203703</v>
       </c>
-      <c r="C25" s="10"/>
+      <c r="C25" s="9">
+        <v>46212.663946967594</v>
+      </c>
       <c r="D25" s="9">
-        <v>46169.85897216435</v>
+        <v>46212.66394828704</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I25" s="9">
         <v>46155</v>
@@ -3056,13 +3064,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O25" s="10" t="s">
         <v>102</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
@@ -3073,12 +3081,12 @@
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B26" s="5">
         <v>46146.78709759259</v>
@@ -3090,16 +3098,16 @@
         <v>46195.92635861111</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I26" s="5">
         <v>46153</v>
@@ -3120,7 +3128,7 @@
         <v>93</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>93</v>
@@ -3143,7 +3151,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B27" s="9">
         <v>46146.78710313658</v>
@@ -3155,16 +3163,16 @@
         <v>46195.92632960648</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I27" s="9">
         <v>46153</v>
@@ -3182,13 +3190,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>74</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
@@ -3199,12 +3207,12 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B28" s="5">
         <v>46146.787108969904</v>
@@ -3216,16 +3224,16 @@
         <v>46195.9263380787</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I28" s="5">
         <v>46155</v>
@@ -3243,13 +3251,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3260,12 +3268,12 @@
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B29" s="9">
         <v>46146.78711427083</v>
@@ -3277,16 +3285,16 @@
         <v>46203.71001635416</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I29" s="9">
         <v>46153</v>
@@ -3307,7 +3315,7 @@
         <v>93</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>93</v>
@@ -3330,7 +3338,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B30" s="5">
         <v>46146.78711935185</v>
@@ -3342,16 +3350,16 @@
         <v>46203.70991413195</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I30" s="5">
         <v>46153</v>
@@ -3369,13 +3377,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>68</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3386,12 +3394,12 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B31" s="9">
         <v>46146.78712466435</v>
@@ -3403,16 +3411,16 @@
         <v>46203.70997798612</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I31" s="9">
         <v>46162</v>
@@ -3430,13 +3438,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
@@ -3447,12 +3455,12 @@
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B32" s="5">
         <v>46146.78712987268</v>
@@ -3464,16 +3472,16 @@
         <v>46203.709962685185</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I32" s="5">
         <v>46161</v>
@@ -3491,13 +3499,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3508,12 +3516,12 @@
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B33" s="9">
         <v>46146.78718802083</v>
@@ -3525,16 +3533,16 @@
         <v>46205.606630173614</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I33" s="9">
         <v>46181</v>
@@ -3555,7 +3563,7 @@
         <v>93</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>93</v>
@@ -3578,7 +3586,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B34" s="5">
         <v>46146.78719326389</v>
@@ -3590,16 +3598,16 @@
         <v>46205.60655203703</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I34" s="5">
         <v>46181</v>
@@ -3617,13 +3625,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>78</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
@@ -3634,12 +3642,12 @@
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B35" s="9">
         <v>46146.78719805555</v>
@@ -3651,16 +3659,16 @@
         <v>46205.60660486111</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I35" s="9">
         <v>46183</v>
@@ -3678,13 +3686,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
@@ -3695,12 +3703,12 @@
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B36" s="5">
         <v>46146.78721570602</v>
@@ -3712,16 +3720,16 @@
         <v>46205.60686332176</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I36" s="5">
         <v>46181</v>
@@ -3742,7 +3750,7 @@
         <v>93</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3765,7 +3773,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B37" s="9">
         <v>46146.787218854166</v>
@@ -3783,10 +3791,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I37" s="9">
         <v>46181</v>
@@ -3804,13 +3812,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>84</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3820,7 +3828,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B38" s="5">
         <v>46146.78722290509</v>
@@ -3832,16 +3840,16 @@
         <v>46205.60683582176</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I38" s="5">
         <v>46183</v>
@@ -3859,13 +3867,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>85</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3875,7 +3883,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B39" s="9">
         <v>46146.78722673611</v>
@@ -3887,16 +3895,16 @@
         <v>46210.16859381944</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I39" s="9">
         <v>46181</v>
@@ -3917,7 +3925,7 @@
         <v>93</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>26</v>
@@ -3929,7 +3937,7 @@
         <v>46217</v>
       </c>
       <c r="S39" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="T39" s="10">
         <v>1</v>
@@ -3940,7 +3948,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B40" s="5">
         <v>46146.787229884256</v>
@@ -3958,10 +3966,10 @@
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I40" s="5">
         <v>46181</v>
@@ -3979,13 +3987,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>90</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -3995,7 +4003,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B41" s="9">
         <v>46146.787233807874</v>
@@ -4007,16 +4015,16 @@
         <v>46205.5916524537</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I41" s="9">
         <v>46188</v>
@@ -4034,13 +4042,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>91</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -4050,7 +4058,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B42" s="5">
         <v>46146.92145594908</v>
@@ -4062,16 +4070,16 @@
         <v>46205.59169479167</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I42" s="6"/>
       <c r="J42" s="5">
@@ -4087,10 +4095,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -4103,7 +4111,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B43" s="9">
         <v>46146.78723741898</v>
@@ -4115,16 +4123,16 @@
         <v>46205.60740758102</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I43" s="9">
         <v>46181</v>
@@ -4145,7 +4153,7 @@
         <v>93</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -4168,7 +4176,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B44" s="5">
         <v>46146.78724063658</v>
@@ -4186,10 +4194,10 @@
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I44" s="5">
         <v>46181</v>
@@ -4207,13 +4215,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>87</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4223,7 +4231,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B45" s="9">
         <v>46146.78724467593</v>
@@ -4235,16 +4243,16 @@
         <v>46205.607379733796</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I45" s="9">
         <v>46183</v>
@@ -4262,13 +4270,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O45" s="10" t="s">
         <v>88</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4278,7 +4286,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B46" s="5">
         <v>46146.78688576389</v>
@@ -4290,7 +4298,7 @@
         <v>46210.52859619213</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4314,7 +4322,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4331,7 +4339,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B47" s="9">
         <v>46146.78724949074</v>
@@ -4343,16 +4351,16 @@
         <v>46197.711020393515</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I47" s="9">
         <v>46156</v>
@@ -4370,13 +4378,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>61</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Q47" s="9">
         <v>46156</v>
@@ -4396,7 +4404,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B48" s="5">
         <v>46146.7872546412</v>
@@ -4408,16 +4416,16 @@
         <v>46203.71488673611</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I48" s="5">
         <v>46169</v>
@@ -4435,13 +4443,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q48" s="5">
         <v>46169</v>
@@ -4461,7 +4469,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B49" s="9">
         <v>46146.787260625</v>
@@ -4479,10 +4487,10 @@
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="9">
@@ -4498,13 +4506,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="Q49" s="9">
         <v>46176</v>
@@ -4524,7 +4532,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B50" s="5">
         <v>46146.78727884259</v>
@@ -4534,16 +4542,16 @@
         <v>46146.93970905093</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I50" s="6"/>
       <c r="J50" s="5">
@@ -4559,10 +4567,10 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4580,12 +4588,12 @@
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B51" s="9">
         <v>46146.78728261574</v>
@@ -4595,16 +4603,16 @@
         <v>46146.939574814816</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="9">
@@ -4620,13 +4628,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="O51" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q51" s="10"/>
       <c r="R51" s="10"/>
@@ -4636,7 +4644,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B52" s="5">
         <v>46146.787286527775</v>
@@ -4646,16 +4654,16 @@
         <v>46146.939575474535</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I52" s="6"/>
       <c r="J52" s="5">
@@ -4671,13 +4679,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
@@ -4687,7 +4695,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B53" s="9">
         <v>46146.787341759264</v>
@@ -4697,7 +4705,7 @@
         <v>46200.68378381945</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>25</v>
@@ -4721,7 +4729,7 @@
         <v>26</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P53" s="10" t="s">
         <v>26</v>
@@ -4731,7 +4739,7 @@
       <c r="S53" s="10"/>
       <c r="T53" s="10"/>
       <c r="U53" s="12" t="s">
-        <v>199</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4773,10 +4781,10 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>204</v>
@@ -4794,7 +4802,7 @@
         <v>1</v>
       </c>
       <c r="U54" s="12" t="s">
-        <v>199</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
@@ -4817,10 +4825,10 @@
         <v>26</v>
       </c>
       <c r="G55" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H55" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" s="9">
@@ -4836,7 +4844,7 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O55" s="10" t="s">
         <v>207</v>
@@ -4899,10 +4907,10 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>211</v>
@@ -4920,7 +4928,7 @@
         <v>0</v>
       </c>
       <c r="U56" s="12" t="s">
-        <v>199</v>
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4943,10 +4951,10 @@
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I57" s="9">
         <v>46192</v>
@@ -4964,7 +4972,7 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O57" s="10" t="s">
         <v>210</v>
@@ -5027,10 +5035,10 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>217</v>
@@ -5048,7 +5056,7 @@
         <v>0</v>
       </c>
       <c r="U58" s="12" t="s">
-        <v>199</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -5071,10 +5079,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I59" s="9">
         <v>46192</v>
@@ -5092,7 +5100,7 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O59" s="10" t="s">
         <v>216</v>
@@ -5539,10 +5547,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I67" s="10"/>
       <c r="J67" s="9">
@@ -5579,7 +5587,7 @@
         <v>1</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>199</v>
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5602,10 +5610,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="5">
@@ -5655,10 +5663,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I69" s="10"/>
       <c r="J69" s="9">
@@ -5697,10 +5705,10 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46146.92121962963</v>
+        <v>46212.664260949074</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>25</v>
@@ -5733,7 +5741,9 @@
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
       <c r="T70" s="6"/>
-      <c r="U70" s="6"/>
+      <c r="U70" s="12" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
@@ -5742,9 +5752,11 @@
       <c r="B71" s="9">
         <v>46146.787437465275</v>
       </c>
-      <c r="C71" s="10"/>
+      <c r="C71" s="9">
+        <v>46212.66404712963</v>
+      </c>
       <c r="D71" s="9">
-        <v>46191.78551768519</v>
+        <v>46212.66406818287</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>250</v>
@@ -5772,10 +5784,10 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P71" s="10" t="s">
         <v>251</v>
@@ -5790,10 +5802,10 @@
         <v>33</v>
       </c>
       <c r="T71" s="10">
-        <v>0</v>
-      </c>
-      <c r="U71" s="12" t="s">
-        <v>199</v>
+        <v>1</v>
+      </c>
+      <c r="U71" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5803,9 +5815,11 @@
       <c r="B72" s="5">
         <v>46146.78744341435</v>
       </c>
-      <c r="C72" s="6"/>
+      <c r="C72" s="5">
+        <v>46212.66403994213</v>
+      </c>
       <c r="D72" s="5">
-        <v>46157.18259200231</v>
+        <v>46212.66405451389</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>253</v>
@@ -5833,10 +5847,10 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>254</v>
@@ -5851,10 +5865,10 @@
         <v>33</v>
       </c>
       <c r="T72" s="6">
-        <v>0</v>
-      </c>
-      <c r="U72" s="11" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="U72" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5864,9 +5878,11 @@
       <c r="B73" s="9">
         <v>46146.7874489699</v>
       </c>
-      <c r="C73" s="10"/>
+      <c r="C73" s="9">
+        <v>46212.66424371528</v>
+      </c>
       <c r="D73" s="9">
-        <v>46203.70999737269</v>
+        <v>46212.664260694444</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>256</v>
@@ -5894,10 +5910,10 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P73" s="10" t="s">
         <v>251</v>
@@ -5912,10 +5928,10 @@
         <v>33</v>
       </c>
       <c r="T73" s="10">
-        <v>0</v>
-      </c>
-      <c r="U73" s="12" t="s">
-        <v>199</v>
+        <v>1</v>
+      </c>
+      <c r="U73" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5955,10 +5971,10 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P74" s="6" t="s">
         <v>259</v>
@@ -5970,13 +5986,13 @@
         <v>46218</v>
       </c>
       <c r="S74" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="T74" s="6">
         <v>0</v>
       </c>
       <c r="U74" s="12" t="s">
-        <v>199</v>
+        <v>95</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -6105,7 +6121,7 @@
         <v>46210.66987453704</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>26</v>
@@ -6160,7 +6176,7 @@
         <v>46210.66993231481</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
@@ -6243,7 +6259,7 @@
         <v>261</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P79" s="10" t="s">
         <v>261</v>
@@ -6275,10 +6291,10 @@
         <v>46197.58893424769</v>
       </c>
       <c r="D80" s="5">
-        <v>46203.71494715278</v>
+        <v>46212.66404658565</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
@@ -6328,10 +6344,10 @@
         <v>46197.58900142361</v>
       </c>
       <c r="D81" s="9">
-        <v>46203.71494597222</v>
+        <v>46212.66404525463</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
@@ -6414,7 +6430,7 @@
         <v>261</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>261</v>
@@ -6446,10 +6462,10 @@
         <v>46210.66999793981</v>
       </c>
       <c r="D83" s="9">
-        <v>46210.66999954861</v>
+        <v>46212.66405841435</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
@@ -6499,10 +6515,10 @@
         <v>46210.67007324074</v>
       </c>
       <c r="D84" s="5">
-        <v>46210.670075243055</v>
+        <v>46212.664059675924</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
@@ -6583,7 +6599,7 @@
         <v>261</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P85" s="10" t="s">
         <v>261</v>
@@ -6615,10 +6631,10 @@
         <v>46210.67028576389</v>
       </c>
       <c r="D86" s="5">
-        <v>46210.67028814815</v>
+        <v>46212.664253379626</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
@@ -6668,10 +6684,10 @@
         <v>46210.67029284722</v>
       </c>
       <c r="D87" s="9">
-        <v>46210.67029388889</v>
+        <v>46212.6642540625</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
@@ -6750,7 +6766,7 @@
         <v>261</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P88" s="6" t="s">
         <v>261</v>
@@ -6768,7 +6784,7 @@
         <v>0</v>
       </c>
       <c r="U88" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -6783,7 +6799,7 @@
         <v>46210.670293460644</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>26</v>
@@ -6811,7 +6827,7 @@
         <v>289</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P89" s="10" t="s">
         <v>291</v>
@@ -6834,7 +6850,7 @@
         <v>46210.67030641204</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
@@ -6862,7 +6878,7 @@
         <v>289</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P90" s="6" t="s">
         <v>291</v>
@@ -6913,7 +6929,7 @@
         <v>261</v>
       </c>
       <c r="O91" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P91" s="10" t="s">
         <v>295</v>
@@ -6931,7 +6947,7 @@
         <v>0</v>
       </c>
       <c r="U91" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
@@ -6946,7 +6962,7 @@
         <v>46146.94244866898</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
@@ -6974,7 +6990,7 @@
         <v>294</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P92" s="6" t="s">
         <v>297</v>
@@ -6997,7 +7013,7 @@
         <v>46146.94244559028</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
@@ -7025,7 +7041,7 @@
         <v>294</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P93" s="10" t="s">
         <v>297</v>
@@ -7141,7 +7157,7 @@
         <v>0</v>
       </c>
       <c r="U95" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
@@ -7156,7 +7172,7 @@
         <v>46146.942643194445</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
@@ -7184,7 +7200,7 @@
         <v>303</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P96" s="6" t="s">
         <v>308</v>
@@ -7207,7 +7223,7 @@
         <v>46146.94264393518</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
@@ -7235,7 +7251,7 @@
         <v>303</v>
       </c>
       <c r="O97" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P97" s="10" t="s">
         <v>310</v>
@@ -7286,7 +7302,7 @@
         <v>300</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P98" s="6" t="s">
         <v>300</v>
@@ -7304,7 +7320,7 @@
         <v>0</v>
       </c>
       <c r="U98" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -7319,7 +7335,7 @@
         <v>46146.94285763889</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F99" s="10" t="s">
         <v>26</v>
@@ -7347,7 +7363,7 @@
         <v>312</v>
       </c>
       <c r="O99" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P99" s="10" t="s">
         <v>314</v>
@@ -7370,7 +7386,7 @@
         <v>46146.94285530093</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
@@ -7398,7 +7414,7 @@
         <v>312</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P100" s="6" t="s">
         <v>316</v>
@@ -7449,7 +7465,7 @@
         <v>300</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P101" s="10" t="s">
         <v>300</v>
@@ -7467,7 +7483,7 @@
         <v>0</v>
       </c>
       <c r="U101" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
@@ -7482,7 +7498,7 @@
         <v>46146.94342792824</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
@@ -7510,7 +7526,7 @@
         <v>318</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P102" s="6" t="s">
         <v>320</v>
@@ -7533,7 +7549,7 @@
         <v>46146.94346471065</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
@@ -7561,7 +7577,7 @@
         <v>318</v>
       </c>
       <c r="O103" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P103" s="10" t="s">
         <v>322</v>
@@ -7612,7 +7628,7 @@
         <v>300</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P104" s="6" t="s">
         <v>325</v>
@@ -7630,7 +7646,7 @@
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7645,7 +7661,7 @@
         <v>46146.94332239583</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>26</v>
@@ -7673,7 +7689,7 @@
         <v>324</v>
       </c>
       <c r="O105" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P105" s="10" t="s">
         <v>324</v>
@@ -7696,7 +7712,7 @@
         <v>46146.943319872684</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
@@ -7724,7 +7740,7 @@
         <v>324</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P106" s="6" t="s">
         <v>324</v>
@@ -7842,7 +7858,7 @@
         <v>0</v>
       </c>
       <c r="U108" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
@@ -7905,7 +7921,7 @@
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-09 19:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="342">
   <si>
     <t>50001543 - ZITRON COLOMBIA EGM</t>
   </si>
@@ -379,348 +379,354 @@
     <t xml:space="preserve">rodete OT 4309,Motor OT 4309,Materiales corte Laser OT 4309,Alabe OT 4309 </t>
   </si>
   <si>
+    <t>1214511244996574</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alabe OT 4309 </t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4309,Generación OC Alabe OT 4309</t>
+  </si>
+  <si>
+    <t>1214511244996589</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4309</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Alabe OT 4309,Alabe OT 4309 </t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
+  </si>
+  <si>
+    <t>1214511142420461</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4309</t>
+  </si>
+  <si>
+    <t>Alabe OT 4309 ,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1214511142420479</t>
+  </si>
+  <si>
+    <t>rodete OT 4309</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete OT 4309,Generación OC Rodete OT 4309</t>
+  </si>
+  <si>
+    <t>1214511240948634</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete OT 4309</t>
+  </si>
+  <si>
+    <t>rodete OT 4309,Fabricación Rodete OT 4309</t>
+  </si>
+  <si>
+    <t>1214511240948652</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete OT 4309</t>
+  </si>
+  <si>
+    <t>rodete OT 4309,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1214511142420756</t>
+  </si>
+  <si>
+    <t>Motor OT 4309</t>
+  </si>
+  <si>
+    <t>Generación OC motor OT 4309,Fabricación motor OT 4309,Planos motor proveedor OT 4309</t>
+  </si>
+  <si>
+    <t>1214511142420771</t>
+  </si>
+  <si>
+    <t>Generación OC motor OT 4309</t>
+  </si>
+  <si>
+    <t>Motor OT 4309,Fabricación motor OT 4309,Planos motor proveedor OT 4309</t>
+  </si>
+  <si>
+    <t>1214511155826380</t>
+  </si>
+  <si>
+    <t>Fabricación motor OT 4309</t>
+  </si>
+  <si>
+    <t>Motor OT 4309,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1214511155826398</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor OT 4309</t>
+  </si>
+  <si>
+    <t>Motor OT 4309,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1214511240963370</t>
+  </si>
+  <si>
+    <t>Materiales corte Laser OT 4309</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC materiales corte Laser OT 4309,Fabricacion Corte Laser  OT 4309</t>
+  </si>
+  <si>
+    <t>1214511240963385</t>
+  </si>
+  <si>
+    <t>Generación OC materiales corte Laser OT 4309</t>
+  </si>
+  <si>
+    <t>Materiales corte Laser OT 4309,Fabricacion Corte Laser  OT 4309</t>
+  </si>
+  <si>
+    <t>1214511245068713</t>
+  </si>
+  <si>
+    <t>Fabricacion Corte Laser  OT 4309</t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser,Materiales corte Laser OT 4309</t>
+  </si>
+  <si>
+    <t>1214511199002704</t>
+  </si>
+  <si>
+    <t>Materiales Corte Plasma  OT 4309</t>
+  </si>
+  <si>
+    <t>Fabricación Corte Plasma OT 4309 ,Generación OC Corte Plasma  OT 4309</t>
+  </si>
+  <si>
+    <t>1214511199002714</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materiales Corte Plasma  OT 4309,Fabricación Corte Plasma OT 4309 </t>
+  </si>
+  <si>
+    <t>1214511199002729</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Corte Plasma OT 4309 </t>
+  </si>
+  <si>
+    <t>Materiales Corte Plasma  OT 4309,Recepcion Materiales corte plasma</t>
+  </si>
+  <si>
+    <t>1214511142484065</t>
+  </si>
+  <si>
+    <t>Fabricación Externa  OT 4309</t>
+  </si>
+  <si>
+    <t>Rosemary Singh</t>
+  </si>
+  <si>
+    <t>rosemary.singh@zitron.com</t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación Externa OT 4309,Fabricación estructura proveedor externo OT 4309</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>1214511142484075</t>
+  </si>
+  <si>
+    <t>Fabricación Externa  OT 4309,Fabricación estructura proveedor externo OT 4309</t>
+  </si>
+  <si>
+    <t>1214511240973505</t>
+  </si>
+  <si>
+    <t>Fabricación estructura proveedor externo OT 4309</t>
+  </si>
+  <si>
+    <t>Control de calidad fabricación externa  OT 4309,Recepcion fabricación externa ,Fabricación Externa  OT 4309</t>
+  </si>
+  <si>
+    <t>1214508463084879</t>
+  </si>
+  <si>
+    <t>Control de calidad fabricación externa  OT 4309</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t>1214511240973520</t>
+  </si>
+  <si>
+    <t>Mecanizado OT 4309</t>
+  </si>
+  <si>
+    <t>Generación OC Mecanizado OT 4309,Fabricación Mecanizado OT 4309</t>
+  </si>
+  <si>
+    <t>1214511240973530</t>
+  </si>
+  <si>
+    <t>Mecanizado OT 4309,Fabricación Mecanizado OT 4309</t>
+  </si>
+  <si>
+    <t>1214511199027682</t>
+  </si>
+  <si>
+    <t>Fabricación Mecanizado OT 4309</t>
+  </si>
+  <si>
+    <t>Mecanizado OT 4309,Recepcion mecanizado</t>
+  </si>
+  <si>
+    <t>1214508463084764</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseñoo:</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1214511199027697</t>
+  </si>
+  <si>
+    <t>Planos preliminar</t>
+  </si>
+  <si>
+    <t>Gonzalo Javier Dávila Bade</t>
+  </si>
+  <si>
+    <t>gonzalo.davila@zitron.com</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseñoo:,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1214511199035045</t>
+  </si>
+  <si>
+    <t>Planos definitivos</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos motor proveedor OT 4309</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseñoo:,check planos</t>
+  </si>
+  <si>
+    <t>1214511240985139</t>
+  </si>
+  <si>
+    <t>Hernan Roberto Gutierrez Barrientos</t>
+  </si>
+  <si>
+    <t>hgutierrez@zitron.com</t>
+  </si>
+  <si>
+    <t>OT 4309 - ZVN 1-9-75/2,OT  4309- ZVN 1-9-75/2,OT 4309 - ZVN 1-9-75/2,OT 4309 - ZVN 1-9-75/2,Propuesta Fabricación externa OT 4309 ,ZVN 1-9-75/2,propuesta Corte Laser OT 4309,Propuesta Corte plasma  OT 4309,Propuesta Mecanizado OT 4309,ZVN 1-9-75/2,ZVN 1-9-75/2,ZVN 1-9-75/2,ZVN 1-9-75/2,ZVN 1-9-75/2</t>
+  </si>
+  <si>
+    <t>1214511155901576</t>
+  </si>
+  <si>
+    <t>check pruebas FAT</t>
+  </si>
+  <si>
+    <t>Francisca González Cornejo</t>
+  </si>
+  <si>
+    <t>francisca.gonzalez@zitron.com</t>
+  </si>
+  <si>
+    <t>ZVN 1-9-75/2,ZVN 1-9-75/2</t>
+  </si>
+  <si>
+    <t>1214511155901586</t>
+  </si>
+  <si>
+    <t>ZVN 1-9-75/2</t>
+  </si>
+  <si>
+    <t>ot 4309- ZVN 1-9-75/2</t>
+  </si>
+  <si>
+    <t>check pruebas FAT,ot 4309- ZVN 1-9-75/2</t>
+  </si>
+  <si>
+    <t>1214511155901596</t>
+  </si>
+  <si>
+    <t>ot 4309 - ZVN 1-9-75/2</t>
+  </si>
+  <si>
+    <t>1214511155796713</t>
+  </si>
+  <si>
+    <t>Bodega:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepcion materiales corte laser,Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>1214511155796723</t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bodega:,Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>1214511245146577</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser,Recepcion Materiales corte plasma</t>
+  </si>
+  <si>
+    <t>OT 4309 - ZVN 1-9-75/2,OT 4309 - ZVN 1-9-75/2,Bodega:</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
   </si>
   <si>
-    <t>1214511244996574</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alabe OT 4309 </t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4309,Generación OC Alabe OT 4309</t>
-  </si>
-  <si>
-    <t>1214511244996589</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4309</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Alabe OT 4309,Alabe OT 4309 </t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214511142420461</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4309</t>
-  </si>
-  <si>
-    <t>Alabe OT 4309 ,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1214511142420479</t>
-  </si>
-  <si>
-    <t>rodete OT 4309</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete OT 4309,Generación OC Rodete OT 4309</t>
-  </si>
-  <si>
-    <t>1214511240948634</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete OT 4309</t>
-  </si>
-  <si>
-    <t>rodete OT 4309,Fabricación Rodete OT 4309</t>
-  </si>
-  <si>
-    <t>1214511240948652</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete OT 4309</t>
-  </si>
-  <si>
-    <t>rodete OT 4309,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1214511142420756</t>
-  </si>
-  <si>
-    <t>Motor OT 4309</t>
-  </si>
-  <si>
-    <t>Generación OC motor OT 4309,Fabricación motor OT 4309,Planos motor proveedor OT 4309</t>
-  </si>
-  <si>
-    <t>1214511142420771</t>
-  </si>
-  <si>
-    <t>Generación OC motor OT 4309</t>
-  </si>
-  <si>
-    <t>Motor OT 4309,Fabricación motor OT 4309,Planos motor proveedor OT 4309</t>
-  </si>
-  <si>
-    <t>1214511155826380</t>
-  </si>
-  <si>
-    <t>Fabricación motor OT 4309</t>
-  </si>
-  <si>
-    <t>Motor OT 4309,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1214511155826398</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor OT 4309</t>
-  </si>
-  <si>
-    <t>Motor OT 4309,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1214511240963370</t>
-  </si>
-  <si>
-    <t>Materiales corte Laser OT 4309</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC materiales corte Laser OT 4309,Fabricacion Corte Laser  OT 4309</t>
-  </si>
-  <si>
-    <t>1214511240963385</t>
-  </si>
-  <si>
-    <t>Generación OC materiales corte Laser OT 4309</t>
-  </si>
-  <si>
-    <t>Materiales corte Laser OT 4309,Fabricacion Corte Laser  OT 4309</t>
-  </si>
-  <si>
-    <t>1214511245068713</t>
-  </si>
-  <si>
-    <t>Fabricacion Corte Laser  OT 4309</t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser,Materiales corte Laser OT 4309</t>
-  </si>
-  <si>
-    <t>1214511199002704</t>
-  </si>
-  <si>
-    <t>Materiales Corte Plasma  OT 4309</t>
-  </si>
-  <si>
-    <t>Fabricación Corte Plasma OT 4309 ,Generación OC Corte Plasma  OT 4309</t>
-  </si>
-  <si>
-    <t>1214511199002714</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Materiales Corte Plasma  OT 4309,Fabricación Corte Plasma OT 4309 </t>
-  </si>
-  <si>
-    <t>1214511199002729</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Corte Plasma OT 4309 </t>
-  </si>
-  <si>
-    <t>Materiales Corte Plasma  OT 4309,Recepcion Materiales corte plasma</t>
-  </si>
-  <si>
-    <t>1214511142484065</t>
-  </si>
-  <si>
-    <t>Fabricación Externa  OT 4309</t>
-  </si>
-  <si>
-    <t>Rosemary Singh</t>
-  </si>
-  <si>
-    <t>rosemary.singh@zitron.com</t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación Externa OT 4309,Fabricación estructura proveedor externo OT 4309</t>
-  </si>
-  <si>
-    <t>Media</t>
-  </si>
-  <si>
-    <t>1214511142484075</t>
-  </si>
-  <si>
-    <t>Fabricación Externa  OT 4309,Fabricación estructura proveedor externo OT 4309</t>
-  </si>
-  <si>
-    <t>1214511240973505</t>
-  </si>
-  <si>
-    <t>Fabricación estructura proveedor externo OT 4309</t>
-  </si>
-  <si>
-    <t>Control de calidad fabricación externa  OT 4309,Recepcion fabricación externa ,Fabricación Externa  OT 4309</t>
-  </si>
-  <si>
-    <t>1214508463084879</t>
-  </si>
-  <si>
-    <t>Control de calidad fabricación externa  OT 4309</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t>1214511240973520</t>
-  </si>
-  <si>
-    <t>Mecanizado OT 4309</t>
-  </si>
-  <si>
-    <t>Generación OC Mecanizado OT 4309,Fabricación Mecanizado OT 4309</t>
-  </si>
-  <si>
-    <t>1214511240973530</t>
-  </si>
-  <si>
-    <t>Mecanizado OT 4309,Fabricación Mecanizado OT 4309</t>
-  </si>
-  <si>
-    <t>1214511199027682</t>
-  </si>
-  <si>
-    <t>Fabricación Mecanizado OT 4309</t>
-  </si>
-  <si>
-    <t>Mecanizado OT 4309,Recepcion mecanizado</t>
-  </si>
-  <si>
-    <t>1214508463084764</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseñoo:</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1214511199027697</t>
-  </si>
-  <si>
-    <t>Planos preliminar</t>
-  </si>
-  <si>
-    <t>Gonzalo Javier Dávila Bade</t>
-  </si>
-  <si>
-    <t>gonzalo.davila@zitron.com</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseñoo:,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1214511199035045</t>
-  </si>
-  <si>
-    <t>Planos definitivos</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos motor proveedor OT 4309</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseñoo:,check planos</t>
-  </si>
-  <si>
-    <t>1214511240985139</t>
-  </si>
-  <si>
-    <t>Hernan Roberto Gutierrez Barrientos</t>
-  </si>
-  <si>
-    <t>hgutierrez@zitron.com</t>
-  </si>
-  <si>
-    <t>OT 4309 - ZVN 1-9-75/2,OT  4309- ZVN 1-9-75/2,OT 4309 - ZVN 1-9-75/2,OT 4309 - ZVN 1-9-75/2,Propuesta Fabricación externa OT 4309 ,ZVN 1-9-75/2,propuesta Corte Laser OT 4309,Propuesta Corte plasma  OT 4309,Propuesta Mecanizado OT 4309,ZVN 1-9-75/2,ZVN 1-9-75/2,ZVN 1-9-75/2,ZVN 1-9-75/2,ZVN 1-9-75/2</t>
-  </si>
-  <si>
-    <t>1214511155901576</t>
-  </si>
-  <si>
-    <t>check pruebas FAT</t>
-  </si>
-  <si>
-    <t>Francisca González Cornejo</t>
-  </si>
-  <si>
-    <t>francisca.gonzalez@zitron.com</t>
-  </si>
-  <si>
-    <t>ZVN 1-9-75/2,ZVN 1-9-75/2</t>
-  </si>
-  <si>
-    <t>1214511155901586</t>
-  </si>
-  <si>
-    <t>ZVN 1-9-75/2</t>
-  </si>
-  <si>
-    <t>check pruebas FAT,ZVN 1-9-75/2</t>
-  </si>
-  <si>
-    <t>1214511155901596</t>
-  </si>
-  <si>
-    <t>1214511155796713</t>
-  </si>
-  <si>
-    <t>Bodega:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recepcion materiales corte laser,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>1214511155796723</t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bodega:,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>1214511245146577</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser,Recepcion Materiales corte plasma</t>
-  </si>
-  <si>
-    <t>OT 4309 - ZVN 1-9-75/2,OT 4309 - ZVN 1-9-75/2,Bodega:</t>
-  </si>
-  <si>
     <t>1214511155961778</t>
   </si>
   <si>
@@ -949,7 +955,7 @@
     <t>Recepcion motor,check planos</t>
   </si>
   <si>
-    <t>Montaje motor,ZVN 1-9-75/2</t>
+    <t>Montaje motor,ot 4309- ZVN 1-9-75/2</t>
   </si>
   <si>
     <t>1214511241215787</t>
@@ -958,12 +964,18 @@
     <t>check planos,Recepcion motor</t>
   </si>
   <si>
+    <t>Montaje motor,ot 4309 - ZVN 1-9-75/2</t>
+  </si>
+  <si>
     <t>1214511241247725</t>
   </si>
   <si>
     <t>Pruebas FAT</t>
   </si>
   <si>
+    <t>ot 4309- ZVN 1-9-75/2,ot 4309 - ZVN 1-9-75/2</t>
+  </si>
+  <si>
     <t>1214511241247740</t>
   </si>
   <si>
@@ -979,13 +991,16 @@
     <t>RE-PINTADO</t>
   </si>
   <si>
+    <t>ot 4309- ZVN 1-9-75/2,ot 4309- ZVN 1-9-75/2</t>
+  </si>
+  <si>
     <t>Montaje:,Coordinacion Entrega con Cliente</t>
   </si>
   <si>
     <t>1214511245386084</t>
   </si>
   <si>
-    <t>RE-PINTADO,ZVN 1-9-75/2</t>
+    <t>RE-PINTADO,ot 4309- ZVN 1-9-75/2</t>
   </si>
   <si>
     <t>1214511245386099</t>
@@ -1012,19 +1027,19 @@
     <t>kpinto@zitron.com</t>
   </si>
   <si>
-    <t>ZVN 1-9-75/2,RE-PINTADO,ZVN 1-9-75/2</t>
+    <t>ot 4309- ZVN 1-9-75/2,RE-PINTADO,ot 4309- ZVN 1-9-75/2</t>
   </si>
   <si>
     <t>1214511245412281</t>
   </si>
   <si>
-    <t>Coordinacion Entrega con Cliente,ZVN 1-9-75/2</t>
+    <t>Coordinacion Entrega con Cliente,ot 4309- ZVN 1-9-75/2</t>
   </si>
   <si>
     <t>1214511241300240</t>
   </si>
   <si>
-    <t>ZVN 1-9-75/2,Coordinacion Entrega con Cliente</t>
+    <t>ot 4309- ZVN 1-9-75/2,Coordinacion Entrega con Cliente</t>
   </si>
   <si>
     <t>1214511245415624</t>
@@ -1036,13 +1051,13 @@
     <t>1214511245415639</t>
   </si>
   <si>
-    <t>ZVN 1-9-75/2,Embalaje</t>
+    <t>ot 4309- ZVN 1-9-75/2,Embalaje</t>
   </si>
   <si>
     <t>1214511245415654</t>
   </si>
   <si>
-    <t>Embalaje,ZVN 1-9-75/2</t>
+    <t>Embalaje,ot 4309- ZVN 1-9-75/2</t>
   </si>
   <si>
     <t>1214511156219005</t>
@@ -1054,13 +1069,13 @@
     <t>1214511241390749</t>
   </si>
   <si>
-    <t>PACKING LIST,Planos Preliminar,ZVN 1-9-75/2</t>
+    <t>PACKING LIST,Planos Preliminar,ot 4309- ZVN 1-9-75/2</t>
   </si>
   <si>
     <t>1214511241390769</t>
   </si>
   <si>
-    <t>Planos Preliminar,PACKING LIST,ZVN 1-9-75/2</t>
+    <t>Planos Preliminar,PACKING LIST,ot 4309- ZVN 1-9-75/2</t>
   </si>
   <si>
     <t>1214511142894089</t>
@@ -2855,9 +2870,11 @@
       <c r="B22" s="5">
         <v>46146.786881064814</v>
       </c>
-      <c r="C22" s="6"/>
+      <c r="C22" s="5">
+        <v>46212.77674577547</v>
+      </c>
       <c r="D22" s="5">
-        <v>46212.66398305555</v>
+        <v>46212.77676006945</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>93</v>
@@ -2892,14 +2909,16 @@
       <c r="Q22" s="6"/>
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
-      <c r="T22" s="6"/>
-      <c r="U22" s="12" t="s">
-        <v>95</v>
+      <c r="T22" s="6">
+        <v>1</v>
+      </c>
+      <c r="U22" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B23" s="9">
         <v>46146.78708193287</v>
@@ -2911,16 +2930,16 @@
         <v>46212.66397574074</v>
       </c>
       <c r="E23" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="10" t="s">
+      <c r="H23" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="I23" s="9">
         <v>46153</v>
@@ -2941,7 +2960,7 @@
         <v>93</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P23" s="10" t="s">
         <v>93</v>
@@ -2964,7 +2983,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B24" s="5">
         <v>46146.78708679398</v>
@@ -2976,16 +2995,16 @@
         <v>46212.663913888886</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="I24" s="5">
         <v>46153</v>
@@ -3003,29 +3022,29 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>71</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T24" s="6">
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B25" s="9">
         <v>46146.78709203703</v>
@@ -3037,16 +3056,16 @@
         <v>46212.66394828704</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="I25" s="9">
         <v>46155</v>
@@ -3064,29 +3083,29 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T25" s="10">
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B26" s="5">
         <v>46146.78709759259</v>
@@ -3098,16 +3117,16 @@
         <v>46195.92635861111</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="I26" s="5">
         <v>46153</v>
@@ -3128,7 +3147,7 @@
         <v>93</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>93</v>
@@ -3151,7 +3170,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B27" s="9">
         <v>46146.78710313658</v>
@@ -3163,16 +3182,16 @@
         <v>46195.92632960648</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="I27" s="9">
         <v>46153</v>
@@ -3190,29 +3209,29 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>74</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
       <c r="S27" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T27" s="10">
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B28" s="5">
         <v>46146.787108969904</v>
@@ -3224,16 +3243,16 @@
         <v>46195.9263380787</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="I28" s="5">
         <v>46155</v>
@@ -3251,29 +3270,29 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
       <c r="S28" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T28" s="6">
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B29" s="9">
         <v>46146.78711427083</v>
@@ -3285,16 +3304,16 @@
         <v>46203.71001635416</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="I29" s="9">
         <v>46153</v>
@@ -3315,7 +3334,7 @@
         <v>93</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>93</v>
@@ -3338,7 +3357,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B30" s="5">
         <v>46146.78711935185</v>
@@ -3350,16 +3369,16 @@
         <v>46203.70991413195</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="I30" s="5">
         <v>46153</v>
@@ -3377,29 +3396,29 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>68</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B31" s="9">
         <v>46146.78712466435</v>
@@ -3411,16 +3430,16 @@
         <v>46203.70997798612</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="I31" s="9">
         <v>46162</v>
@@ -3438,29 +3457,29 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
       <c r="S31" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T31" s="10">
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B32" s="5">
         <v>46146.78712987268</v>
@@ -3472,16 +3491,16 @@
         <v>46203.709962685185</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="I32" s="5">
         <v>46161</v>
@@ -3499,29 +3518,29 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B33" s="9">
         <v>46146.78718802083</v>
@@ -3533,16 +3552,16 @@
         <v>46205.606630173614</v>
       </c>
       <c r="E33" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G33" s="10" t="s">
+      <c r="H33" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="I33" s="9">
         <v>46181</v>
@@ -3563,7 +3582,7 @@
         <v>93</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>93</v>
@@ -3586,7 +3605,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B34" s="5">
         <v>46146.78719326389</v>
@@ -3598,16 +3617,16 @@
         <v>46205.60655203703</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>132</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>133</v>
       </c>
       <c r="I34" s="5">
         <v>46181</v>
@@ -3625,29 +3644,29 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>78</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B35" s="9">
         <v>46146.78719805555</v>
@@ -3659,16 +3678,16 @@
         <v>46205.60660486111</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="I35" s="9">
         <v>46183</v>
@@ -3686,29 +3705,29 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
       <c r="S35" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T35" s="10">
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B36" s="5">
         <v>46146.78721570602</v>
@@ -3720,16 +3739,16 @@
         <v>46205.60686332176</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>132</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>133</v>
       </c>
       <c r="I36" s="5">
         <v>46181</v>
@@ -3750,7 +3769,7 @@
         <v>93</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3773,7 +3792,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B37" s="9">
         <v>46146.787218854166</v>
@@ -3791,10 +3810,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="I37" s="9">
         <v>46181</v>
@@ -3812,13 +3831,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>84</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3828,7 +3847,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B38" s="5">
         <v>46146.78722290509</v>
@@ -3840,16 +3859,16 @@
         <v>46205.60683582176</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>132</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>133</v>
       </c>
       <c r="I38" s="5">
         <v>46183</v>
@@ -3867,13 +3886,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>85</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3883,7 +3902,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B39" s="9">
         <v>46146.78722673611</v>
@@ -3895,16 +3914,16 @@
         <v>46210.16859381944</v>
       </c>
       <c r="E39" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G39" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G39" s="10" t="s">
+      <c r="H39" s="10" t="s">
         <v>151</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>152</v>
       </c>
       <c r="I39" s="9">
         <v>46181</v>
@@ -3925,7 +3944,7 @@
         <v>93</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>26</v>
@@ -3937,7 +3956,7 @@
         <v>46217</v>
       </c>
       <c r="S39" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="T39" s="10">
         <v>1</v>
@@ -3948,7 +3967,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B40" s="5">
         <v>46146.787229884256</v>
@@ -3966,10 +3985,10 @@
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>151</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="I40" s="5">
         <v>46181</v>
@@ -3987,13 +4006,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>90</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -4003,7 +4022,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B41" s="9">
         <v>46146.787233807874</v>
@@ -4015,16 +4034,16 @@
         <v>46205.5916524537</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="H41" s="10" t="s">
         <v>151</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>152</v>
       </c>
       <c r="I41" s="9">
         <v>46188</v>
@@ -4042,13 +4061,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>91</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -4058,7 +4077,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B42" s="5">
         <v>46146.92145594908</v>
@@ -4070,16 +4089,16 @@
         <v>46205.59169479167</v>
       </c>
       <c r="E42" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G42" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G42" s="6" t="s">
+      <c r="H42" s="6" t="s">
         <v>162</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>163</v>
       </c>
       <c r="I42" s="6"/>
       <c r="J42" s="5">
@@ -4095,10 +4114,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -4111,7 +4130,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B43" s="9">
         <v>46146.78723741898</v>
@@ -4123,16 +4142,16 @@
         <v>46205.60740758102</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="I43" s="9">
         <v>46181</v>
@@ -4153,7 +4172,7 @@
         <v>93</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -4176,7 +4195,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B44" s="5">
         <v>46146.78724063658</v>
@@ -4194,10 +4213,10 @@
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>132</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>133</v>
       </c>
       <c r="I44" s="5">
         <v>46181</v>
@@ -4215,13 +4234,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>87</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4231,7 +4250,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B45" s="9">
         <v>46146.78724467593</v>
@@ -4243,16 +4262,16 @@
         <v>46205.607379733796</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="H45" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="I45" s="9">
         <v>46183</v>
@@ -4270,13 +4289,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="O45" s="10" t="s">
         <v>88</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4286,7 +4305,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B46" s="5">
         <v>46146.78688576389</v>
@@ -4298,7 +4317,7 @@
         <v>46210.52859619213</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4322,7 +4341,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4339,7 +4358,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B47" s="9">
         <v>46146.78724949074</v>
@@ -4351,16 +4370,16 @@
         <v>46197.711020393515</v>
       </c>
       <c r="E47" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" s="10" t="s">
+      <c r="H47" s="10" t="s">
         <v>177</v>
-      </c>
-      <c r="H47" s="10" t="s">
-        <v>178</v>
       </c>
       <c r="I47" s="9">
         <v>46156</v>
@@ -4378,13 +4397,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>61</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q47" s="9">
         <v>46156</v>
@@ -4404,7 +4423,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B48" s="5">
         <v>46146.7872546412</v>
@@ -4416,16 +4435,16 @@
         <v>46203.71488673611</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>178</v>
       </c>
       <c r="I48" s="5">
         <v>46169</v>
@@ -4443,13 +4462,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="O48" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="P48" s="6" t="s">
         <v>182</v>
-      </c>
-      <c r="P48" s="6" t="s">
-        <v>183</v>
       </c>
       <c r="Q48" s="5">
         <v>46169</v>
@@ -4469,7 +4488,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B49" s="9">
         <v>46146.787260625</v>
@@ -4487,10 +4506,10 @@
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="H49" s="10" t="s">
         <v>185</v>
-      </c>
-      <c r="H49" s="10" t="s">
-        <v>186</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="9">
@@ -4506,13 +4525,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Q49" s="9">
         <v>46176</v>
@@ -4532,7 +4551,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B50" s="5">
         <v>46146.78727884259</v>
@@ -4542,16 +4561,16 @@
         <v>46146.93970905093</v>
       </c>
       <c r="E50" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G50" s="6" t="s">
+      <c r="H50" s="6" t="s">
         <v>190</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="I50" s="6"/>
       <c r="J50" s="5">
@@ -4567,10 +4586,10 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4582,18 +4601,18 @@
         <v>46232</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B51" s="9">
         <v>46146.78728261574</v>
@@ -4603,16 +4622,16 @@
         <v>46146.939574814816</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="H51" s="10" t="s">
         <v>190</v>
-      </c>
-      <c r="H51" s="10" t="s">
-        <v>191</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="9">
@@ -4628,7 +4647,7 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="O51" s="10" t="s">
         <v>194</v>
@@ -4654,16 +4673,16 @@
         <v>46146.939575474535</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="H52" s="6" t="s">
         <v>190</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="I52" s="6"/>
       <c r="J52" s="5">
@@ -4679,10 +4698,10 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>195</v>
@@ -4695,17 +4714,19 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B53" s="9">
         <v>46146.787341759264</v>
       </c>
-      <c r="C53" s="10"/>
+      <c r="C53" s="9">
+        <v>46212.77632917824</v>
+      </c>
       <c r="D53" s="9">
-        <v>46200.68378381945</v>
+        <v>46212.77634790509</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>25</v>
@@ -4729,7 +4750,7 @@
         <v>26</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P53" s="10" t="s">
         <v>26</v>
@@ -4737,33 +4758,37 @@
       <c r="Q53" s="10"/>
       <c r="R53" s="10"/>
       <c r="S53" s="10"/>
-      <c r="T53" s="10"/>
-      <c r="U53" s="12" t="s">
-        <v>95</v>
+      <c r="T53" s="10">
+        <v>1</v>
+      </c>
+      <c r="U53" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B54" s="5">
         <v>46146.787345254634</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46212.77629162037</v>
+      </c>
       <c r="D54" s="5">
-        <v>46205.60662056713</v>
+        <v>46212.77630914352</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I54" s="5">
         <v>46190</v>
@@ -4781,13 +4806,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Q54" s="5">
         <v>46190</v>
@@ -4801,13 +4826,13 @@
       <c r="T54" s="6">
         <v>1</v>
       </c>
-      <c r="U54" s="12" t="s">
-        <v>95</v>
+      <c r="U54" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B55" s="9">
         <v>46146.787358877315</v>
@@ -4816,19 +4841,19 @@
         <v>46200.68377538194</v>
       </c>
       <c r="D55" s="9">
-        <v>46200.6837771412</v>
+        <v>46212.776321666664</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H55" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="H55" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" s="9">
@@ -4844,13 +4869,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P55" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q55" s="9">
         <v>46192</v>
@@ -4864,32 +4889,34 @@
       <c r="T55" s="10">
         <v>1</v>
       </c>
-      <c r="U55" s="7" t="s">
-        <v>27</v>
+      <c r="U55" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B56" s="5">
         <v>46146.78735064815</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46212.77630217593</v>
+      </c>
       <c r="D56" s="5">
-        <v>46205.606852488425</v>
+        <v>46212.77631554398</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I56" s="5">
         <v>46190</v>
@@ -4907,13 +4934,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="Q56" s="5">
         <v>46190</v>
@@ -4925,15 +4952,15 @@
         <v>33</v>
       </c>
       <c r="T56" s="6">
-        <v>0</v>
-      </c>
-      <c r="U56" s="12" t="s">
-        <v>95</v>
+        <v>1</v>
+      </c>
+      <c r="U56" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B57" s="9">
         <v>46146.79730351851</v>
@@ -4942,19 +4969,19 @@
         <v>46200.68386630787</v>
       </c>
       <c r="D57" s="9">
-        <v>46200.683887164356</v>
+        <v>46212.776320439814</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H57" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="H57" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="I57" s="9">
         <v>46192</v>
@@ -4972,13 +4999,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="Q57" s="9">
         <v>46192</v>
@@ -4992,32 +5019,34 @@
       <c r="T57" s="10">
         <v>1</v>
       </c>
-      <c r="U57" s="7" t="s">
-        <v>27</v>
+      <c r="U57" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B58" s="5">
         <v>46146.78735449074</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46212.77631068287</v>
+      </c>
       <c r="D58" s="5">
-        <v>46205.607397581014</v>
+        <v>46212.77632949074</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I58" s="5">
         <v>46190</v>
@@ -5035,13 +5064,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="Q58" s="5">
         <v>46190</v>
@@ -5053,15 +5082,15 @@
         <v>33</v>
       </c>
       <c r="T58" s="6">
-        <v>0</v>
-      </c>
-      <c r="U58" s="12" t="s">
-        <v>95</v>
+        <v>1</v>
+      </c>
+      <c r="U58" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B59" s="9">
         <v>46146.79750996528</v>
@@ -5070,19 +5099,19 @@
         <v>46200.68395946759</v>
       </c>
       <c r="D59" s="9">
-        <v>46200.68397615741</v>
+        <v>46212.77632611111</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H59" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="H59" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="I59" s="9">
         <v>46192</v>
@@ -5100,13 +5129,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O59" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="P59" s="10" t="s">
         <v>216</v>
-      </c>
-      <c r="P59" s="10" t="s">
-        <v>214</v>
       </c>
       <c r="Q59" s="9">
         <v>46192</v>
@@ -5120,13 +5149,13 @@
       <c r="T59" s="10">
         <v>1</v>
       </c>
-      <c r="U59" s="7" t="s">
-        <v>27</v>
+      <c r="U59" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B60" s="5">
         <v>46146.787364398144</v>
@@ -5138,7 +5167,7 @@
         <v>46200.68337925926</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>25</v>
@@ -5162,7 +5191,7 @@
         <v>26</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>26</v>
@@ -5179,7 +5208,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B61" s="9">
         <v>46146.78736695602</v>
@@ -5191,16 +5220,16 @@
         <v>46198.89361756944</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I61" s="9">
         <v>46195</v>
@@ -5218,13 +5247,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Q61" s="9">
         <v>46195</v>
@@ -5244,7 +5273,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B62" s="5">
         <v>46146.79438380787</v>
@@ -5256,16 +5285,16 @@
         <v>46200.6839671412</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I62" s="5">
         <v>46195</v>
@@ -5283,13 +5312,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="Q62" s="6"/>
       <c r="R62" s="6"/>
@@ -5299,7 +5328,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B63" s="9">
         <v>46146.79440119213</v>
@@ -5311,16 +5340,16 @@
         <v>46200.683967916666</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I63" s="9">
         <v>46195</v>
@@ -5338,13 +5367,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Q63" s="10"/>
       <c r="R63" s="10"/>
@@ -5354,7 +5383,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B64" s="5">
         <v>46146.78737179398</v>
@@ -5366,16 +5395,16 @@
         <v>46205.203211134256</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I64" s="5">
         <v>46198</v>
@@ -5393,13 +5422,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Q64" s="5">
         <v>46198</v>
@@ -5419,7 +5448,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B65" s="9">
         <v>46146.78737561342</v>
@@ -5431,16 +5460,16 @@
         <v>46203.71492597222</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H65" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I65" s="9">
         <v>46198</v>
@@ -5458,13 +5487,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O65" s="10" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="P65" s="10" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="Q65" s="10"/>
       <c r="R65" s="10"/>
@@ -5474,7 +5503,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B66" s="5">
         <v>46146.78738193287</v>
@@ -5486,16 +5515,16 @@
         <v>46203.714927361114</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I66" s="5">
         <v>46198</v>
@@ -5513,13 +5542,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="Q66" s="6"/>
       <c r="R66" s="6"/>
@@ -5529,7 +5558,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B67" s="9">
         <v>46146.78740461805</v>
@@ -5541,16 +5570,16 @@
         <v>46206.20677265046</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H67" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="I67" s="10"/>
       <c r="J67" s="9">
@@ -5566,13 +5595,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Q67" s="9">
         <v>46205</v>
@@ -5587,12 +5616,12 @@
         <v>1</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>95</v>
+        <v>210</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B68" s="5">
         <v>46146.787408564815</v>
@@ -5604,16 +5633,16 @@
         <v>46203.7149283912</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>162</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>163</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="5">
@@ -5629,13 +5658,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="Q68" s="6"/>
       <c r="R68" s="6"/>
@@ -5645,7 +5674,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B69" s="9">
         <v>46146.78741372685</v>
@@ -5657,16 +5686,16 @@
         <v>46203.714929317124</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H69" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="H69" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="I69" s="10"/>
       <c r="J69" s="9">
@@ -5682,13 +5711,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="O69" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="P69" s="10" t="s">
         <v>246</v>
-      </c>
-      <c r="P69" s="10" t="s">
-        <v>244</v>
       </c>
       <c r="Q69" s="10"/>
       <c r="R69" s="10"/>
@@ -5698,17 +5727,19 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B70" s="5">
         <v>46146.78743457176</v>
       </c>
-      <c r="C70" s="6"/>
+      <c r="C70" s="5">
+        <v>46212.77656946759</v>
+      </c>
       <c r="D70" s="5">
-        <v>46212.664260949074</v>
+        <v>46212.776581342594</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>25</v>
@@ -5732,7 +5763,7 @@
         <v>26</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>26</v>
@@ -5740,14 +5771,16 @@
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
-      <c r="T70" s="6"/>
-      <c r="U70" s="12" t="s">
-        <v>95</v>
+      <c r="T70" s="6">
+        <v>1</v>
+      </c>
+      <c r="U70" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B71" s="9">
         <v>46146.787437465275</v>
@@ -5759,16 +5792,16 @@
         <v>46212.66406818287</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I71" s="10"/>
       <c r="J71" s="9">
@@ -5784,13 +5817,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Q71" s="9">
         <v>46175</v>
@@ -5810,7 +5843,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B72" s="5">
         <v>46146.78744341435</v>
@@ -5822,16 +5855,16 @@
         <v>46212.66405451389</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I72" s="6"/>
       <c r="J72" s="5">
@@ -5847,13 +5880,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="Q72" s="5">
         <v>46156</v>
@@ -5873,7 +5906,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B73" s="9">
         <v>46146.7874489699</v>
@@ -5885,16 +5918,16 @@
         <v>46212.664260694444</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I73" s="10"/>
       <c r="J73" s="9">
@@ -5910,13 +5943,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Q73" s="9">
         <v>46191</v>
@@ -5936,26 +5969,28 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B74" s="5">
         <v>46146.78746039352</v>
       </c>
-      <c r="C74" s="6"/>
+      <c r="C74" s="5">
+        <v>46212.77655145833</v>
+      </c>
       <c r="D74" s="5">
-        <v>46211.19095658565</v>
+        <v>46212.776568009256</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
@@ -5971,13 +6006,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="Q74" s="5">
         <v>46218</v>
@@ -5986,18 +6021,18 @@
         <v>46218</v>
       </c>
       <c r="S74" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="T74" s="6">
-        <v>0</v>
-      </c>
-      <c r="U74" s="12" t="s">
-        <v>95</v>
+        <v>1</v>
+      </c>
+      <c r="U74" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B75" s="9">
         <v>46146.78750452546</v>
@@ -6007,7 +6042,7 @@
         <v>46210.67031722222</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>25</v>
@@ -6031,7 +6066,7 @@
         <v>26</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="P75" s="10" t="s">
         <v>26</v>
@@ -6044,7 +6079,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B76" s="5">
         <v>46146.787508912035</v>
@@ -6053,10 +6088,10 @@
         <v>46210.669946180555</v>
       </c>
       <c r="D76" s="5">
-        <v>46210.669961203705</v>
+        <v>46212.776568437504</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
@@ -6083,13 +6118,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="Q76" s="5">
         <v>46219</v>
@@ -6098,18 +6133,18 @@
         <v>46225</v>
       </c>
       <c r="S76" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T76" s="6">
         <v>1</v>
       </c>
-      <c r="U76" s="7" t="s">
-        <v>27</v>
+      <c r="U76" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B77" s="9">
         <v>46146.78752016203</v>
@@ -6118,10 +6153,10 @@
         <v>46210.66987290509</v>
       </c>
       <c r="D77" s="9">
-        <v>46210.66987453704</v>
+        <v>46212.77656100695</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>26</v>
@@ -6148,10 +6183,10 @@
         <v>26</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="P77" s="10" t="s">
         <v>26</v>
@@ -6164,7 +6199,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B78" s="5">
         <v>46146.78752439815</v>
@@ -6173,10 +6208,10 @@
         <v>46210.66993070602</v>
       </c>
       <c r="D78" s="5">
-        <v>46210.66993231481</v>
+        <v>46212.7765616088</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
@@ -6203,10 +6238,10 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>26</v>
@@ -6219,7 +6254,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B79" s="9">
         <v>46146.78758131944</v>
@@ -6231,7 +6266,7 @@
         <v>46197.5890270949</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>26</v>
@@ -6256,13 +6291,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="Q79" s="9">
         <v>46226</v>
@@ -6271,7 +6306,7 @@
         <v>46226</v>
       </c>
       <c r="S79" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T79" s="10">
         <v>1</v>
@@ -6282,7 +6317,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B80" s="5">
         <v>46146.78758657408</v>
@@ -6294,7 +6329,7 @@
         <v>46212.66404658565</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
@@ -6319,13 +6354,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="Q80" s="6"/>
       <c r="R80" s="6"/>
@@ -6335,7 +6370,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B81" s="9">
         <v>46146.787592939814</v>
@@ -6347,7 +6382,7 @@
         <v>46212.66404525463</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
@@ -6372,13 +6407,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="10" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="Q81" s="10"/>
       <c r="R81" s="10"/>
@@ -6388,7 +6423,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B82" s="5">
         <v>46146.78761755787</v>
@@ -6400,7 +6435,7 @@
         <v>46210.670105150464</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6427,13 +6462,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="Q82" s="5">
         <v>46227</v>
@@ -6442,7 +6477,7 @@
         <v>46227</v>
       </c>
       <c r="S82" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T82" s="6">
         <v>1</v>
@@ -6453,7 +6488,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B83" s="9">
         <v>46146.78762708334</v>
@@ -6465,7 +6500,7 @@
         <v>46212.66405841435</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
@@ -6490,13 +6525,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="10" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="O83" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="P83" s="10" t="s">
         <v>279</v>
-      </c>
-      <c r="P83" s="10" t="s">
-        <v>277</v>
       </c>
       <c r="Q83" s="10"/>
       <c r="R83" s="10"/>
@@ -6506,7 +6541,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B84" s="5">
         <v>46146.78763331019</v>
@@ -6518,7 +6553,7 @@
         <v>46212.664059675924</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
@@ -6543,13 +6578,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="O84" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="P84" s="6" t="s">
         <v>279</v>
-      </c>
-      <c r="P84" s="6" t="s">
-        <v>277</v>
       </c>
       <c r="Q84" s="6"/>
       <c r="R84" s="6"/>
@@ -6559,7 +6594,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B85" s="9">
         <v>46146.78769865741</v>
@@ -6571,7 +6606,7 @@
         <v>46210.67032010417</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>26</v>
@@ -6596,13 +6631,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="Q85" s="9">
         <v>46230</v>
@@ -6611,7 +6646,7 @@
         <v>46230</v>
       </c>
       <c r="S85" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T85" s="10">
         <v>1</v>
@@ -6622,7 +6657,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B86" s="5">
         <v>46146.787703553244</v>
@@ -6634,7 +6669,7 @@
         <v>46212.664253379626</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
@@ -6659,13 +6694,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="Q86" s="6"/>
       <c r="R86" s="6"/>
@@ -6675,7 +6710,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B87" s="9">
         <v>46146.78770892361</v>
@@ -6687,7 +6722,7 @@
         <v>46212.6642540625</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
@@ -6712,13 +6747,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="10" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="Q87" s="10"/>
       <c r="R87" s="10"/>
@@ -6728,7 +6763,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B88" s="5">
         <v>46146.78773052084</v>
@@ -6738,7 +6773,7 @@
         <v>46146.94197813657</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
@@ -6763,13 +6798,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>192</v>
+        <v>293</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="Q88" s="5">
         <v>46231</v>
@@ -6778,25 +6813,25 @@
         <v>46231</v>
       </c>
       <c r="S88" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T88" s="6">
         <v>0</v>
       </c>
       <c r="U88" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B89" s="9">
         <v>46146.78773511574</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="9">
-        <v>46210.670293460644</v>
+        <v>46212.77709833333</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>194</v>
@@ -6824,13 +6859,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="10" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="Q89" s="10"/>
       <c r="R89" s="10"/>
@@ -6840,17 +6875,17 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="B90" s="5">
         <v>46146.78774035879</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46210.67030641204</v>
+        <v>46212.777147280096</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
@@ -6875,13 +6910,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="Q90" s="6"/>
       <c r="R90" s="6"/>
@@ -6891,7 +6926,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B91" s="9">
         <v>46146.787759479164</v>
@@ -6901,7 +6936,7 @@
         <v>46146.94197326389</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
@@ -6926,13 +6961,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O91" s="10" t="s">
-        <v>192</v>
+        <v>299</v>
       </c>
       <c r="P91" s="10" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="Q91" s="9">
         <v>46233</v>
@@ -6941,25 +6976,25 @@
         <v>46233</v>
       </c>
       <c r="S91" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T91" s="10">
         <v>0</v>
       </c>
       <c r="U91" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B92" s="5">
         <v>46146.78776425926</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46146.94244866898</v>
+        <v>46212.77733467593</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>194</v>
@@ -6987,13 +7022,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="Q92" s="6"/>
       <c r="R92" s="6"/>
@@ -7003,14 +7038,14 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="B93" s="9">
         <v>46146.787768587965</v>
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46146.94244559028</v>
+        <v>46212.77735347222</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>194</v>
@@ -7038,13 +7073,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="Q93" s="10"/>
       <c r="R93" s="10"/>
@@ -7054,7 +7089,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B94" s="5">
         <v>46146.78778571759</v>
@@ -7064,7 +7099,7 @@
         <v>46146.9405634838</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>25</v>
@@ -7088,7 +7123,7 @@
         <v>26</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="P94" s="6" t="s">
         <v>26</v>
@@ -7101,7 +7136,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B95" s="9">
         <v>46146.78778912037</v>
@@ -7111,16 +7146,16 @@
         <v>46146.9429809375</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="10" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="H95" s="10" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="9">
@@ -7136,13 +7171,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="Q95" s="9">
         <v>46234</v>
@@ -7151,25 +7186,25 @@
         <v>46234</v>
       </c>
       <c r="S95" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T95" s="10">
         <v>0</v>
       </c>
       <c r="U95" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B96" s="5">
         <v>46146.78779429398</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46146.942643194445</v>
+        <v>46212.77737873842</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>194</v>
@@ -7178,10 +7213,10 @@
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="5">
@@ -7197,13 +7232,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="O96" s="6" t="s">
         <v>194</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -7213,14 +7248,14 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B97" s="9">
         <v>46146.787798414356</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46146.94264393518</v>
+        <v>46212.777400127314</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>194</v>
@@ -7229,10 +7264,10 @@
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="H97" s="10" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="9">
@@ -7248,13 +7283,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="O97" s="10" t="s">
         <v>194</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Q97" s="10"/>
       <c r="R97" s="10"/>
@@ -7264,7 +7299,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B98" s="5">
         <v>46146.787814745374</v>
@@ -7274,7 +7309,7 @@
         <v>46146.94289535879</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7299,13 +7334,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>192</v>
+        <v>299</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="Q98" s="5">
         <v>46237</v>
@@ -7314,25 +7349,25 @@
         <v>46237</v>
       </c>
       <c r="S98" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T98" s="6">
         <v>0</v>
       </c>
       <c r="U98" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B99" s="9">
         <v>46146.78781900463</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46146.94285763889</v>
+        <v>46212.777429884256</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>194</v>
@@ -7360,13 +7395,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="10" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="O99" s="10" t="s">
         <v>194</v>
       </c>
       <c r="P99" s="10" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="Q99" s="10"/>
       <c r="R99" s="10"/>
@@ -7376,14 +7411,14 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B100" s="5">
         <v>46146.787823148145</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46146.94285530093</v>
+        <v>46212.77744148148</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>194</v>
@@ -7411,13 +7446,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="O100" s="6" t="s">
         <v>194</v>
       </c>
       <c r="P100" s="6" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7427,7 +7462,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="B101" s="9">
         <v>46146.787891527776</v>
@@ -7437,16 +7472,16 @@
         <v>46146.9431597338</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H101" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I101" s="10"/>
       <c r="J101" s="9">
@@ -7462,13 +7497,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>192</v>
+        <v>299</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="Q101" s="9">
         <v>46238</v>
@@ -7477,25 +7512,25 @@
         <v>46238</v>
       </c>
       <c r="S101" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T101" s="10">
         <v>0</v>
       </c>
       <c r="U101" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B102" s="5">
         <v>46146.78789762731</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46146.94342792824</v>
+        <v>46212.77746881945</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>194</v>
@@ -7504,10 +7539,10 @@
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="5">
@@ -7523,13 +7558,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="O102" s="6" t="s">
         <v>194</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="Q102" s="6"/>
       <c r="R102" s="6"/>
@@ -7539,14 +7574,14 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B103" s="9">
         <v>46146.78790538195</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46146.94346471065</v>
+        <v>46212.77748577546</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>194</v>
@@ -7555,10 +7590,10 @@
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H103" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="9">
@@ -7574,13 +7609,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="10" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="O103" s="10" t="s">
         <v>194</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="Q103" s="10"/>
       <c r="R103" s="10"/>
@@ -7590,7 +7625,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B104" s="5">
         <v>46146.787928171296</v>
@@ -7600,16 +7635,16 @@
         <v>46146.94327527778</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="5">
@@ -7625,13 +7660,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>192</v>
+        <v>299</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="Q104" s="5">
         <v>46239</v>
@@ -7640,25 +7675,25 @@
         <v>46239</v>
       </c>
       <c r="S104" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T104" s="6">
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="B105" s="9">
         <v>46146.787934409724</v>
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="9">
-        <v>46146.94332239583</v>
+        <v>46212.77751017361</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>194</v>
@@ -7667,10 +7702,10 @@
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I105" s="10"/>
       <c r="J105" s="9">
@@ -7686,13 +7721,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="10" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="O105" s="10" t="s">
         <v>194</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="Q105" s="10"/>
       <c r="R105" s="10"/>
@@ -7702,14 +7737,14 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B106" s="5">
         <v>46146.787939131944</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46146.943319872684</v>
+        <v>46212.777535706016</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>194</v>
@@ -7718,10 +7753,10 @@
         <v>26</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I106" s="6"/>
       <c r="J106" s="5">
@@ -7737,13 +7772,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="O106" s="6" t="s">
         <v>194</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7753,7 +7788,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B107" s="9">
         <v>46146.787957974535</v>
@@ -7763,7 +7798,7 @@
         <v>46146.94056351852</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>25</v>
@@ -7787,7 +7822,7 @@
         <v>26</v>
       </c>
       <c r="O107" s="10" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="P107" s="10" t="s">
         <v>26</v>
@@ -7800,7 +7835,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B108" s="5">
         <v>46146.78796153935</v>
@@ -7810,16 +7845,16 @@
         <v>46146.94352958333</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="I108" s="5">
         <v>46240</v>
@@ -7837,13 +7872,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="O108" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="O108" s="6" t="s">
-        <v>324</v>
-      </c>
       <c r="P108" s="6" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="Q108" s="5">
         <v>46240</v>
@@ -7852,18 +7887,18 @@
         <v>46248</v>
       </c>
       <c r="S108" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T108" s="6">
         <v>0</v>
       </c>
       <c r="U108" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B109" s="9">
         <v>46146.78796724537</v>
@@ -7873,7 +7908,7 @@
         <v>46196.86770128472</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>26</v>
@@ -7900,13 +7935,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="O109" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="O109" s="10" t="s">
-        <v>324</v>
-      </c>
       <c r="P109" s="10" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="Q109" s="9">
         <v>46240</v>
@@ -7915,13 +7950,13 @@
         <v>46248</v>
       </c>
       <c r="S109" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T109" s="10">
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-10 16:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="341">
   <si>
     <t>50001543 - ZITRON COLOMBIA EGM</t>
   </si>
@@ -119,30 +119,6 @@
   </si>
   <si>
     <t>Apertura pedido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para el pedido 1466 se deben suministrar 5 unidades ZVN 1-10-126/2 para Zitron Perú (Cía. Minera Poderosa):
-    Fabricación / Planos:
-·         O/4302; Ventilador ZVN 1-10-126/2 con motor WEG.
-·         Alcance: Tobera + Rejilla + Carcasa
-    Selección de Rodete:
-        Rodete de placas s/plano 3073.00
-        Alabe s/ plano 3073.01
-        Z8 N600
-        Código 300003
-        hgutierrez@zitron.com, tu apoyo con la definición de calaje.
-    Tratamiento superficial estándar Zitron:
-        Preparación de superficie: Arenado SSPC-SP10
-        1ª capa imprimación 60 micras Hempadur 15570 Color 12430
-        2ª capa intermedia 40 micras Hempathane HS 55610 Color 20450 RAL 9001 Blanco.
-    Datos eléctricos motor:
-·         Motor WEG 90 kW; 2 Polos; IE3
-·         Frame 280
-·         460V, 60HZ
-·         OC19034: 23-04-2026
-·         Se requiere duplicado de placas.
-    Fecha de entrega: 30-04-2026
-</t>
   </si>
   <si>
     <t>1214511244960122</t>
@@ -1866,7 +1842,7 @@
         <v>46175.87207239583</v>
       </c>
       <c r="D6" s="5">
-        <v>46175.87209802083</v>
+        <v>46213.69123809028</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1888,7 +1864,7 @@
         <v>26</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="M6" s="6" t="s">
         <v>26</v>
@@ -1920,7 +1896,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="9">
         <v>46146.78699966436</v>
@@ -1932,7 +1908,7 @@
         <v>46175.872098576394</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>26</v>
@@ -1951,7 +1927,7 @@
         <v>26</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>26</v>
@@ -1983,7 +1959,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" s="5">
         <v>46146.7870025</v>
@@ -1995,7 +1971,7 @@
         <v>46175.87209884259</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>26</v>
@@ -2014,7 +1990,7 @@
         <v>26</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M8" s="6" t="s">
         <v>26</v>
@@ -2026,7 +2002,7 @@
         <v>26</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q8" s="5">
         <v>46147</v>
@@ -2046,7 +2022,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" s="9">
         <v>46146.787006631945</v>
@@ -2058,7 +2034,7 @@
         <v>46175.87209942129</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>26</v>
@@ -2077,7 +2053,7 @@
         <v>26</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>26</v>
@@ -2109,7 +2085,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="5">
         <v>46146.78687210648</v>
@@ -2121,7 +2097,7 @@
         <v>46197.6494803588</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>25</v>
@@ -2145,7 +2121,7 @@
         <v>26</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P10" s="6" t="s">
         <v>26</v>
@@ -2162,7 +2138,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="9">
         <v>46146.787010162036</v>
@@ -2174,16 +2150,16 @@
         <v>46197.64823298611</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="10" t="s">
+      <c r="H11" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="I11" s="9">
         <v>46147</v>
@@ -2195,19 +2171,19 @@
         <v>26</v>
       </c>
       <c r="L11" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="P11" s="10" t="s">
         <v>54</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="O11" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="P11" s="10" t="s">
-        <v>55</v>
       </c>
       <c r="Q11" s="9">
         <v>46147</v>
@@ -2227,7 +2203,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="5">
         <v>46146.7870155787</v>
@@ -2239,16 +2215,16 @@
         <v>46197.64898236111</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="I12" s="5">
         <v>46147</v>
@@ -2260,19 +2236,19 @@
         <v>26</v>
       </c>
       <c r="L12" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="P12" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N12" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="P12" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="Q12" s="5">
         <v>46147</v>
@@ -2292,7 +2268,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="9">
         <v>46146.787021400465</v>
@@ -2304,16 +2280,16 @@
         <v>46197.6494675463</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="I13" s="9">
         <v>46147</v>
@@ -2325,19 +2301,19 @@
         <v>26</v>
       </c>
       <c r="L13" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O13" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="P13" s="10" t="s">
         <v>62</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N13" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="O13" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>63</v>
       </c>
       <c r="Q13" s="9">
         <v>46147</v>
@@ -2357,7 +2333,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46146.7868765162</v>
@@ -2369,7 +2345,7 @@
         <v>46204.908018587965</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>25</v>
@@ -2393,7 +2369,7 @@
         <v>26</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P14" s="6" t="s">
         <v>26</v>
@@ -2410,7 +2386,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" s="9">
         <v>46146.7870415625</v>
@@ -2422,16 +2398,16 @@
         <v>46203.70941623843</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F15" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="I15" s="9">
         <v>46149</v>
@@ -2449,13 +2425,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Q15" s="9">
         <v>46149</v>
@@ -2475,7 +2451,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B16" s="5">
         <v>46146.78704743055</v>
@@ -2487,16 +2463,16 @@
         <v>46203.70945753472</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="I16" s="5">
         <v>46149</v>
@@ -2514,13 +2490,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Q16" s="5">
         <v>46149</v>
@@ -2540,7 +2516,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B17" s="9">
         <v>46146.78705320602</v>
@@ -2552,16 +2528,16 @@
         <v>46204.907181365736</v>
       </c>
       <c r="E17" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>75</v>
-      </c>
       <c r="H17" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I17" s="9">
         <v>46149</v>
@@ -2579,13 +2555,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Q17" s="9">
         <v>46149</v>
@@ -2605,7 +2581,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B18" s="5">
         <v>46146.78705905093</v>
@@ -2617,16 +2593,16 @@
         <v>46204.90714847222</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G18" s="6" t="s">
+      <c r="H18" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>80</v>
       </c>
       <c r="I18" s="5">
         <v>46177</v>
@@ -2644,13 +2620,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O18" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="P18" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>82</v>
       </c>
       <c r="Q18" s="5">
         <v>46146</v>
@@ -2670,7 +2646,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B19" s="9">
         <v>46146.78706952547</v>
@@ -2682,16 +2658,16 @@
         <v>46204.9075317824</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>79</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>80</v>
       </c>
       <c r="I19" s="9">
         <v>46177</v>
@@ -2709,13 +2685,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="9">
         <v>46177</v>
@@ -2735,7 +2711,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B20" s="5">
         <v>46146.78707340278</v>
@@ -2747,16 +2723,16 @@
         <v>46204.90778255787</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>80</v>
       </c>
       <c r="I20" s="5">
         <v>46177</v>
@@ -2774,13 +2750,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Q20" s="5">
         <v>46177</v>
@@ -2800,7 +2776,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B21" s="9">
         <v>46146.78707737269</v>
@@ -2812,16 +2788,16 @@
         <v>46204.90800618056</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>79</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>80</v>
       </c>
       <c r="I21" s="9">
         <v>46177</v>
@@ -2839,13 +2815,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q21" s="9">
         <v>46177</v>
@@ -2865,7 +2841,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B22" s="5">
         <v>46146.786881064814</v>
@@ -2877,7 +2853,7 @@
         <v>46212.77676006945</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>25</v>
@@ -2901,7 +2877,7 @@
         <v>26</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P22" s="6" t="s">
         <v>26</v>
@@ -2918,7 +2894,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B23" s="9">
         <v>46146.78708193287</v>
@@ -2930,16 +2906,16 @@
         <v>46212.66397574074</v>
       </c>
       <c r="E23" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="10" t="s">
+      <c r="H23" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="I23" s="9">
         <v>46153</v>
@@ -2957,13 +2933,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q23" s="9">
         <v>46153</v>
@@ -2983,7 +2959,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B24" s="5">
         <v>46146.78708679398</v>
@@ -2995,16 +2971,16 @@
         <v>46212.663913888886</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="I24" s="5">
         <v>46153</v>
@@ -3022,29 +2998,29 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T24" s="6">
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B25" s="9">
         <v>46146.78709203703</v>
@@ -3056,16 +3032,16 @@
         <v>46212.66394828704</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="I25" s="9">
         <v>46155</v>
@@ -3083,29 +3059,29 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T25" s="10">
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B26" s="5">
         <v>46146.78709759259</v>
@@ -3117,16 +3093,16 @@
         <v>46195.92635861111</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="I26" s="5">
         <v>46153</v>
@@ -3144,13 +3120,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q26" s="5">
         <v>46153</v>
@@ -3170,7 +3146,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B27" s="9">
         <v>46146.78710313658</v>
@@ -3182,16 +3158,16 @@
         <v>46195.92632960648</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="I27" s="9">
         <v>46153</v>
@@ -3209,29 +3185,29 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
       <c r="S27" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T27" s="10">
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B28" s="5">
         <v>46146.787108969904</v>
@@ -3243,16 +3219,16 @@
         <v>46195.9263380787</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="I28" s="5">
         <v>46155</v>
@@ -3270,29 +3246,29 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
       <c r="S28" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T28" s="6">
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B29" s="9">
         <v>46146.78711427083</v>
@@ -3304,16 +3280,16 @@
         <v>46203.71001635416</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="I29" s="9">
         <v>46153</v>
@@ -3331,13 +3307,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q29" s="9">
         <v>46153</v>
@@ -3357,7 +3333,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B30" s="5">
         <v>46146.78711935185</v>
@@ -3369,16 +3345,16 @@
         <v>46203.70991413195</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="I30" s="5">
         <v>46153</v>
@@ -3396,29 +3372,29 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B31" s="9">
         <v>46146.78712466435</v>
@@ -3430,16 +3406,16 @@
         <v>46203.70997798612</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="I31" s="9">
         <v>46162</v>
@@ -3457,29 +3433,29 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
       <c r="S31" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T31" s="10">
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B32" s="5">
         <v>46146.78712987268</v>
@@ -3491,16 +3467,16 @@
         <v>46203.709962685185</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="I32" s="5">
         <v>46161</v>
@@ -3518,29 +3494,29 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B33" s="9">
         <v>46146.78718802083</v>
@@ -3552,16 +3528,16 @@
         <v>46205.606630173614</v>
       </c>
       <c r="E33" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G33" s="10" t="s">
+      <c r="H33" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>132</v>
       </c>
       <c r="I33" s="9">
         <v>46181</v>
@@ -3579,13 +3555,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P33" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q33" s="9">
         <v>46150</v>
@@ -3605,7 +3581,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B34" s="5">
         <v>46146.78719326389</v>
@@ -3617,16 +3593,16 @@
         <v>46205.60655203703</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="I34" s="5">
         <v>46181</v>
@@ -3644,29 +3620,29 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B35" s="9">
         <v>46146.78719805555</v>
@@ -3678,16 +3654,16 @@
         <v>46205.60660486111</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>132</v>
       </c>
       <c r="I35" s="9">
         <v>46183</v>
@@ -3705,29 +3681,29 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
       <c r="S35" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T35" s="10">
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B36" s="5">
         <v>46146.78721570602</v>
@@ -3739,16 +3715,16 @@
         <v>46205.60686332176</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="I36" s="5">
         <v>46181</v>
@@ -3766,10 +3742,10 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3792,7 +3768,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B37" s="9">
         <v>46146.787218854166</v>
@@ -3804,16 +3780,16 @@
         <v>46205.60679543982</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>132</v>
       </c>
       <c r="I37" s="9">
         <v>46181</v>
@@ -3831,13 +3807,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O37" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3847,7 +3823,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B38" s="5">
         <v>46146.78722290509</v>
@@ -3859,16 +3835,16 @@
         <v>46205.60683582176</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="I38" s="5">
         <v>46183</v>
@@ -3886,13 +3862,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3902,7 +3878,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B39" s="9">
         <v>46146.78722673611</v>
@@ -3914,16 +3890,16 @@
         <v>46210.16859381944</v>
       </c>
       <c r="E39" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G39" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G39" s="10" t="s">
+      <c r="H39" s="10" t="s">
         <v>150</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>151</v>
       </c>
       <c r="I39" s="9">
         <v>46181</v>
@@ -3941,10 +3917,10 @@
         <v>26</v>
       </c>
       <c r="N39" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>26</v>
@@ -3956,7 +3932,7 @@
         <v>46217</v>
       </c>
       <c r="S39" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="T39" s="10">
         <v>1</v>
@@ -3967,7 +3943,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B40" s="5">
         <v>46146.787229884256</v>
@@ -3979,16 +3955,16 @@
         <v>46205.54751966435</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="I40" s="5">
         <v>46181</v>
@@ -4006,13 +3982,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -4022,7 +3998,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B41" s="9">
         <v>46146.787233807874</v>
@@ -4034,16 +4010,16 @@
         <v>46205.5916524537</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="H41" s="10" t="s">
         <v>150</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>151</v>
       </c>
       <c r="I41" s="9">
         <v>46188</v>
@@ -4061,13 +4037,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O41" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -4077,7 +4053,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B42" s="5">
         <v>46146.92145594908</v>
@@ -4089,16 +4065,16 @@
         <v>46205.59169479167</v>
       </c>
       <c r="E42" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G42" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G42" s="6" t="s">
+      <c r="H42" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="I42" s="6"/>
       <c r="J42" s="5">
@@ -4114,10 +4090,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -4130,7 +4106,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B43" s="9">
         <v>46146.78723741898</v>
@@ -4142,16 +4118,16 @@
         <v>46205.60740758102</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>132</v>
       </c>
       <c r="I43" s="9">
         <v>46181</v>
@@ -4169,10 +4145,10 @@
         <v>26</v>
       </c>
       <c r="N43" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -4195,7 +4171,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B44" s="5">
         <v>46146.78724063658</v>
@@ -4207,16 +4183,16 @@
         <v>46205.607340787035</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="I44" s="5">
         <v>46181</v>
@@ -4234,13 +4210,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4250,7 +4226,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B45" s="9">
         <v>46146.78724467593</v>
@@ -4262,16 +4238,16 @@
         <v>46205.607379733796</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H45" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>132</v>
       </c>
       <c r="I45" s="9">
         <v>46183</v>
@@ -4289,13 +4265,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4305,7 +4281,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B46" s="5">
         <v>46146.78688576389</v>
@@ -4317,7 +4293,7 @@
         <v>46210.52859619213</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4341,7 +4317,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4358,7 +4334,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B47" s="9">
         <v>46146.78724949074</v>
@@ -4370,16 +4346,16 @@
         <v>46197.711020393515</v>
       </c>
       <c r="E47" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" s="10" t="s">
+      <c r="H47" s="10" t="s">
         <v>176</v>
-      </c>
-      <c r="H47" s="10" t="s">
-        <v>177</v>
       </c>
       <c r="I47" s="9">
         <v>46156</v>
@@ -4397,13 +4373,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O47" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Q47" s="9">
         <v>46156</v>
@@ -4423,7 +4399,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B48" s="5">
         <v>46146.7872546412</v>
@@ -4435,16 +4411,16 @@
         <v>46203.71488673611</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>177</v>
       </c>
       <c r="I48" s="5">
         <v>46169</v>
@@ -4462,13 +4438,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O48" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="P48" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="P48" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="Q48" s="5">
         <v>46169</v>
@@ -4488,7 +4464,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B49" s="9">
         <v>46146.787260625</v>
@@ -4500,16 +4476,16 @@
         <v>46203.71493509259</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="H49" s="10" t="s">
         <v>184</v>
-      </c>
-      <c r="H49" s="10" t="s">
-        <v>185</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="9">
@@ -4525,13 +4501,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Q49" s="9">
         <v>46176</v>
@@ -4551,7 +4527,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B50" s="5">
         <v>46146.78727884259</v>
@@ -4561,16 +4537,16 @@
         <v>46146.93970905093</v>
       </c>
       <c r="E50" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G50" s="6" t="s">
+      <c r="H50" s="6" t="s">
         <v>189</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>190</v>
       </c>
       <c r="I50" s="6"/>
       <c r="J50" s="5">
@@ -4586,10 +4562,10 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4601,18 +4577,18 @@
         <v>46232</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B51" s="9">
         <v>46146.78728261574</v>
@@ -4622,16 +4598,16 @@
         <v>46146.939574814816</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="H51" s="10" t="s">
         <v>189</v>
-      </c>
-      <c r="H51" s="10" t="s">
-        <v>190</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="9">
@@ -4647,13 +4623,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="O51" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="P51" s="10" t="s">
         <v>194</v>
-      </c>
-      <c r="P51" s="10" t="s">
-        <v>195</v>
       </c>
       <c r="Q51" s="10"/>
       <c r="R51" s="10"/>
@@ -4663,7 +4639,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B52" s="5">
         <v>46146.787286527775</v>
@@ -4673,16 +4649,16 @@
         <v>46146.939575474535</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="H52" s="6" t="s">
         <v>189</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>190</v>
       </c>
       <c r="I52" s="6"/>
       <c r="J52" s="5">
@@ -4698,13 +4674,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
@@ -4714,7 +4690,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B53" s="9">
         <v>46146.787341759264</v>
@@ -4726,7 +4702,7 @@
         <v>46212.77634790509</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>25</v>
@@ -4750,7 +4726,7 @@
         <v>26</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="P53" s="10" t="s">
         <v>26</v>
@@ -4767,7 +4743,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B54" s="5">
         <v>46146.787345254634</v>
@@ -4779,16 +4755,16 @@
         <v>46212.77630914352</v>
       </c>
       <c r="E54" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="F54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G54" s="6" t="s">
+      <c r="H54" s="6" t="s">
         <v>203</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>204</v>
       </c>
       <c r="I54" s="5">
         <v>46190</v>
@@ -4806,13 +4782,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q54" s="5">
         <v>46190</v>
@@ -4832,7 +4808,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B55" s="9">
         <v>46146.787358877315</v>
@@ -4844,16 +4820,16 @@
         <v>46212.776321666664</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="H55" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="H55" s="10" t="s">
-        <v>162</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" s="9">
@@ -4869,13 +4845,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O55" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="P55" s="10" t="s">
         <v>208</v>
-      </c>
-      <c r="P55" s="10" t="s">
-        <v>209</v>
       </c>
       <c r="Q55" s="9">
         <v>46192</v>
@@ -4890,12 +4866,12 @@
         <v>1</v>
       </c>
       <c r="U55" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B56" s="5">
         <v>46146.78735064815</v>
@@ -4907,16 +4883,16 @@
         <v>46212.77631554398</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="H56" s="6" t="s">
         <v>203</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>204</v>
       </c>
       <c r="I56" s="5">
         <v>46190</v>
@@ -4934,13 +4910,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q56" s="5">
         <v>46190</v>
@@ -4960,7 +4936,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B57" s="9">
         <v>46146.79730351851</v>
@@ -4972,16 +4948,16 @@
         <v>46212.776320439814</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="H57" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="H57" s="10" t="s">
-        <v>162</v>
       </c>
       <c r="I57" s="9">
         <v>46192</v>
@@ -4999,13 +4975,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q57" s="9">
         <v>46192</v>
@@ -5020,12 +4996,12 @@
         <v>1</v>
       </c>
       <c r="U57" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B58" s="5">
         <v>46146.78735449074</v>
@@ -5037,16 +5013,16 @@
         <v>46212.77632949074</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>203</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>204</v>
       </c>
       <c r="I58" s="5">
         <v>46190</v>
@@ -5064,13 +5040,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Q58" s="5">
         <v>46190</v>
@@ -5090,7 +5066,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B59" s="9">
         <v>46146.79750996528</v>
@@ -5102,16 +5078,16 @@
         <v>46212.77632611111</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="H59" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="H59" s="10" t="s">
-        <v>162</v>
       </c>
       <c r="I59" s="9">
         <v>46192</v>
@@ -5129,13 +5105,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O59" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q59" s="9">
         <v>46192</v>
@@ -5150,12 +5126,12 @@
         <v>1</v>
       </c>
       <c r="U59" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B60" s="5">
         <v>46146.787364398144</v>
@@ -5167,7 +5143,7 @@
         <v>46200.68337925926</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>25</v>
@@ -5191,7 +5167,7 @@
         <v>26</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>26</v>
@@ -5208,7 +5184,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B61" s="9">
         <v>46146.78736695602</v>
@@ -5220,16 +5196,16 @@
         <v>46198.89361756944</v>
       </c>
       <c r="E61" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="F61" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G61" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="F61" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G61" s="10" t="s">
+      <c r="H61" s="10" t="s">
         <v>226</v>
-      </c>
-      <c r="H61" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="I61" s="9">
         <v>46195</v>
@@ -5247,13 +5223,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Q61" s="9">
         <v>46195</v>
@@ -5273,7 +5249,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B62" s="5">
         <v>46146.79438380787</v>
@@ -5285,16 +5261,16 @@
         <v>46200.6839671412</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="I62" s="5">
         <v>46195</v>
@@ -5312,13 +5288,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="O62" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="P62" s="6" t="s">
         <v>231</v>
-      </c>
-      <c r="P62" s="6" t="s">
-        <v>232</v>
       </c>
       <c r="Q62" s="6"/>
       <c r="R62" s="6"/>
@@ -5328,7 +5304,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B63" s="9">
         <v>46146.79440119213</v>
@@ -5340,16 +5316,16 @@
         <v>46200.683967916666</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H63" s="10" t="s">
         <v>226</v>
-      </c>
-      <c r="H63" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="I63" s="9">
         <v>46195</v>
@@ -5367,13 +5343,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="O63" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="P63" s="10" t="s">
         <v>234</v>
-      </c>
-      <c r="P63" s="10" t="s">
-        <v>235</v>
       </c>
       <c r="Q63" s="10"/>
       <c r="R63" s="10"/>
@@ -5383,7 +5359,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B64" s="5">
         <v>46146.78737179398</v>
@@ -5395,16 +5371,16 @@
         <v>46205.203211134256</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="I64" s="5">
         <v>46198</v>
@@ -5422,13 +5398,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Q64" s="5">
         <v>46198</v>
@@ -5448,7 +5424,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B65" s="9">
         <v>46146.78737561342</v>
@@ -5460,16 +5436,16 @@
         <v>46203.71492597222</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H65" s="10" t="s">
         <v>226</v>
-      </c>
-      <c r="H65" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="I65" s="9">
         <v>46198</v>
@@ -5487,13 +5463,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="O65" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="P65" s="10" t="s">
         <v>240</v>
-      </c>
-      <c r="P65" s="10" t="s">
-        <v>241</v>
       </c>
       <c r="Q65" s="10"/>
       <c r="R65" s="10"/>
@@ -5503,7 +5479,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B66" s="5">
         <v>46146.78738193287</v>
@@ -5515,16 +5491,16 @@
         <v>46203.714927361114</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="I66" s="5">
         <v>46198</v>
@@ -5542,13 +5518,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="O66" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="P66" s="6" t="s">
         <v>240</v>
-      </c>
-      <c r="P66" s="6" t="s">
-        <v>241</v>
       </c>
       <c r="Q66" s="6"/>
       <c r="R66" s="6"/>
@@ -5558,7 +5534,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B67" s="9">
         <v>46146.78740461805</v>
@@ -5570,16 +5546,16 @@
         <v>46206.20677265046</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="H67" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>162</v>
       </c>
       <c r="I67" s="10"/>
       <c r="J67" s="9">
@@ -5595,13 +5571,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Q67" s="9">
         <v>46205</v>
@@ -5616,12 +5592,12 @@
         <v>1</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B68" s="5">
         <v>46146.787408564815</v>
@@ -5633,16 +5609,16 @@
         <v>46203.7149283912</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="5">
@@ -5658,13 +5634,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="Q68" s="6"/>
       <c r="R68" s="6"/>
@@ -5674,7 +5650,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B69" s="9">
         <v>46146.78741372685</v>
@@ -5686,16 +5662,16 @@
         <v>46203.714929317124</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="H69" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="H69" s="10" t="s">
-        <v>162</v>
       </c>
       <c r="I69" s="10"/>
       <c r="J69" s="9">
@@ -5711,13 +5687,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="O69" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="Q69" s="10"/>
       <c r="R69" s="10"/>
@@ -5727,7 +5703,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B70" s="5">
         <v>46146.78743457176</v>
@@ -5739,7 +5715,7 @@
         <v>46212.776581342594</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>25</v>
@@ -5763,7 +5739,7 @@
         <v>26</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>26</v>
@@ -5780,7 +5756,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B71" s="9">
         <v>46146.787437465275</v>
@@ -5792,16 +5768,16 @@
         <v>46212.66406818287</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="H71" s="10" t="s">
         <v>203</v>
-      </c>
-      <c r="H71" s="10" t="s">
-        <v>204</v>
       </c>
       <c r="I71" s="10"/>
       <c r="J71" s="9">
@@ -5817,13 +5793,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="Q71" s="9">
         <v>46175</v>
@@ -5843,7 +5819,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B72" s="5">
         <v>46146.78744341435</v>
@@ -5855,16 +5831,16 @@
         <v>46212.66405451389</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>203</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>204</v>
       </c>
       <c r="I72" s="6"/>
       <c r="J72" s="5">
@@ -5880,13 +5856,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Q72" s="5">
         <v>46156</v>
@@ -5906,7 +5882,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B73" s="9">
         <v>46146.7874489699</v>
@@ -5918,16 +5894,16 @@
         <v>46212.664260694444</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="H73" s="10" t="s">
         <v>203</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>204</v>
       </c>
       <c r="I73" s="10"/>
       <c r="J73" s="9">
@@ -5943,13 +5919,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="Q73" s="9">
         <v>46191</v>
@@ -5969,7 +5945,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B74" s="5">
         <v>46146.78746039352</v>
@@ -5981,16 +5957,16 @@
         <v>46212.776568009256</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>203</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>204</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
@@ -6006,13 +5982,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="Q74" s="5">
         <v>46218</v>
@@ -6021,7 +5997,7 @@
         <v>46218</v>
       </c>
       <c r="S74" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="T74" s="6">
         <v>1</v>
@@ -6032,7 +6008,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B75" s="9">
         <v>46146.78750452546</v>
@@ -6042,7 +6018,7 @@
         <v>46210.67031722222</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>25</v>
@@ -6066,7 +6042,7 @@
         <v>26</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="P75" s="10" t="s">
         <v>26</v>
@@ -6079,7 +6055,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B76" s="5">
         <v>46146.787508912035</v>
@@ -6091,16 +6067,16 @@
         <v>46212.776568437504</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I76" s="5">
         <v>46219</v>
@@ -6118,13 +6094,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Q76" s="5">
         <v>46219</v>
@@ -6133,18 +6109,18 @@
         <v>46225</v>
       </c>
       <c r="S76" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T76" s="6">
         <v>1</v>
       </c>
       <c r="U76" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B77" s="9">
         <v>46146.78752016203</v>
@@ -6156,16 +6132,16 @@
         <v>46212.77656100695</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I77" s="9">
         <v>46219</v>
@@ -6183,10 +6159,10 @@
         <v>26</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="P77" s="10" t="s">
         <v>26</v>
@@ -6199,7 +6175,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B78" s="5">
         <v>46146.78752439815</v>
@@ -6211,16 +6187,16 @@
         <v>46212.7765616088</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I78" s="5">
         <v>46219</v>
@@ -6238,10 +6214,10 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>26</v>
@@ -6254,7 +6230,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B79" s="9">
         <v>46146.78758131944</v>
@@ -6266,16 +6242,16 @@
         <v>46197.5890270949</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H79" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="9">
@@ -6291,13 +6267,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Q79" s="9">
         <v>46226</v>
@@ -6306,7 +6282,7 @@
         <v>46226</v>
       </c>
       <c r="S79" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T79" s="10">
         <v>1</v>
@@ -6317,7 +6293,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B80" s="5">
         <v>46146.78758657408</v>
@@ -6329,16 +6305,16 @@
         <v>46212.66404658565</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I80" s="6"/>
       <c r="J80" s="5">
@@ -6354,13 +6330,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O80" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="P80" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="P80" s="6" t="s">
-        <v>275</v>
       </c>
       <c r="Q80" s="6"/>
       <c r="R80" s="6"/>
@@ -6370,7 +6346,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B81" s="9">
         <v>46146.787592939814</v>
@@ -6382,16 +6358,16 @@
         <v>46212.66404525463</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I81" s="10"/>
       <c r="J81" s="9">
@@ -6407,13 +6383,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="Q81" s="10"/>
       <c r="R81" s="10"/>
@@ -6423,7 +6399,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B82" s="5">
         <v>46146.78761755787</v>
@@ -6435,16 +6411,16 @@
         <v>46210.670105150464</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I82" s="5">
         <v>46227</v>
@@ -6462,13 +6438,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Q82" s="5">
         <v>46227</v>
@@ -6477,7 +6453,7 @@
         <v>46227</v>
       </c>
       <c r="S82" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T82" s="6">
         <v>1</v>
@@ -6488,7 +6464,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B83" s="9">
         <v>46146.78762708334</v>
@@ -6500,16 +6476,16 @@
         <v>46212.66405841435</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I83" s="10"/>
       <c r="J83" s="9">
@@ -6525,13 +6501,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Q83" s="10"/>
       <c r="R83" s="10"/>
@@ -6541,7 +6517,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B84" s="5">
         <v>46146.78763331019</v>
@@ -6553,16 +6529,16 @@
         <v>46212.664059675924</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I84" s="6"/>
       <c r="J84" s="5">
@@ -6578,13 +6554,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Q84" s="6"/>
       <c r="R84" s="6"/>
@@ -6594,7 +6570,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B85" s="9">
         <v>46146.78769865741</v>
@@ -6606,16 +6582,16 @@
         <v>46210.67032010417</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I85" s="10"/>
       <c r="J85" s="9">
@@ -6631,13 +6607,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Q85" s="9">
         <v>46230</v>
@@ -6646,7 +6622,7 @@
         <v>46230</v>
       </c>
       <c r="S85" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T85" s="10">
         <v>1</v>
@@ -6657,7 +6633,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B86" s="5">
         <v>46146.787703553244</v>
@@ -6669,16 +6645,16 @@
         <v>46212.664253379626</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I86" s="6"/>
       <c r="J86" s="5">
@@ -6694,13 +6670,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="O86" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="P86" s="6" t="s">
         <v>286</v>
-      </c>
-      <c r="P86" s="6" t="s">
-        <v>287</v>
       </c>
       <c r="Q86" s="6"/>
       <c r="R86" s="6"/>
@@ -6710,7 +6686,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B87" s="9">
         <v>46146.78770892361</v>
@@ -6722,16 +6698,16 @@
         <v>46212.6642540625</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I87" s="10"/>
       <c r="J87" s="9">
@@ -6747,13 +6723,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="O87" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="P87" s="10" t="s">
         <v>289</v>
-      </c>
-      <c r="P87" s="10" t="s">
-        <v>290</v>
       </c>
       <c r="Q87" s="10"/>
       <c r="R87" s="10"/>
@@ -6763,7 +6739,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B88" s="5">
         <v>46146.78773052084</v>
@@ -6773,16 +6749,16 @@
         <v>46146.94197813657</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="5">
@@ -6798,13 +6774,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Q88" s="5">
         <v>46231</v>
@@ -6813,18 +6789,18 @@
         <v>46231</v>
       </c>
       <c r="S88" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T88" s="6">
         <v>0</v>
       </c>
       <c r="U88" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B89" s="9">
         <v>46146.78773511574</v>
@@ -6834,16 +6810,16 @@
         <v>46212.77709833333</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="9">
@@ -6859,13 +6835,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="Q89" s="10"/>
       <c r="R89" s="10"/>
@@ -6875,7 +6851,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B90" s="5">
         <v>46146.78774035879</v>
@@ -6885,16 +6861,16 @@
         <v>46212.777147280096</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="5">
@@ -6910,13 +6886,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="Q90" s="6"/>
       <c r="R90" s="6"/>
@@ -6926,7 +6902,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B91" s="9">
         <v>46146.787759479164</v>
@@ -6936,16 +6912,16 @@
         <v>46146.94197326389</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H91" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" s="9">
@@ -6961,13 +6937,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O91" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="P91" s="10" t="s">
         <v>299</v>
-      </c>
-      <c r="P91" s="10" t="s">
-        <v>300</v>
       </c>
       <c r="Q91" s="9">
         <v>46233</v>
@@ -6976,18 +6952,18 @@
         <v>46233</v>
       </c>
       <c r="S91" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T91" s="10">
         <v>0</v>
       </c>
       <c r="U91" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B92" s="5">
         <v>46146.78776425926</v>
@@ -6997,16 +6973,16 @@
         <v>46212.77733467593</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I92" s="6"/>
       <c r="J92" s="5">
@@ -7022,13 +6998,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="Q92" s="6"/>
       <c r="R92" s="6"/>
@@ -7038,7 +7014,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B93" s="9">
         <v>46146.787768587965</v>
@@ -7048,16 +7024,16 @@
         <v>46212.77735347222</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G93" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H93" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="9">
@@ -7073,13 +7049,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="Q93" s="10"/>
       <c r="R93" s="10"/>
@@ -7089,7 +7065,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B94" s="5">
         <v>46146.78778571759</v>
@@ -7099,7 +7075,7 @@
         <v>46146.9405634838</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>25</v>
@@ -7123,7 +7099,7 @@
         <v>26</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P94" s="6" t="s">
         <v>26</v>
@@ -7136,7 +7112,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B95" s="9">
         <v>46146.78778912037</v>
@@ -7146,16 +7122,16 @@
         <v>46146.9429809375</v>
       </c>
       <c r="E95" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="F95" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G95" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="F95" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G95" s="10" t="s">
+      <c r="H95" s="10" t="s">
         <v>309</v>
-      </c>
-      <c r="H95" s="10" t="s">
-        <v>310</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="9">
@@ -7171,13 +7147,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="Q95" s="9">
         <v>46234</v>
@@ -7186,18 +7162,18 @@
         <v>46234</v>
       </c>
       <c r="S95" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T95" s="10">
         <v>0</v>
       </c>
       <c r="U95" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B96" s="5">
         <v>46146.78779429398</v>
@@ -7207,16 +7183,16 @@
         <v>46212.77737873842</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="H96" s="6" t="s">
         <v>309</v>
-      </c>
-      <c r="H96" s="6" t="s">
-        <v>310</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="5">
@@ -7232,13 +7208,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -7248,7 +7224,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B97" s="9">
         <v>46146.787798414356</v>
@@ -7258,16 +7234,16 @@
         <v>46212.777400127314</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="H97" s="10" t="s">
         <v>309</v>
-      </c>
-      <c r="H97" s="10" t="s">
-        <v>310</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="9">
@@ -7283,13 +7259,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="O97" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q97" s="10"/>
       <c r="R97" s="10"/>
@@ -7299,7 +7275,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B98" s="5">
         <v>46146.787814745374</v>
@@ -7309,16 +7285,16 @@
         <v>46146.94289535879</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I98" s="6"/>
       <c r="J98" s="5">
@@ -7334,13 +7310,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="Q98" s="5">
         <v>46237</v>
@@ -7349,18 +7325,18 @@
         <v>46237</v>
       </c>
       <c r="S98" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T98" s="6">
         <v>0</v>
       </c>
       <c r="U98" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B99" s="9">
         <v>46146.78781900463</v>
@@ -7370,16 +7346,16 @@
         <v>46212.777429884256</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F99" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H99" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I99" s="10"/>
       <c r="J99" s="9">
@@ -7395,13 +7371,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="10" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="O99" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P99" s="10" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="Q99" s="10"/>
       <c r="R99" s="10"/>
@@ -7411,7 +7387,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B100" s="5">
         <v>46146.787823148145</v>
@@ -7421,16 +7397,16 @@
         <v>46212.77744148148</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I100" s="6"/>
       <c r="J100" s="5">
@@ -7446,13 +7422,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P100" s="6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7462,7 +7438,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B101" s="9">
         <v>46146.787891527776</v>
@@ -7472,16 +7448,16 @@
         <v>46146.9431597338</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H101" s="10" t="s">
         <v>226</v>
-      </c>
-      <c r="H101" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="I101" s="10"/>
       <c r="J101" s="9">
@@ -7497,13 +7473,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="Q101" s="9">
         <v>46238</v>
@@ -7512,18 +7488,18 @@
         <v>46238</v>
       </c>
       <c r="S101" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T101" s="10">
         <v>0</v>
       </c>
       <c r="U101" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B102" s="5">
         <v>46146.78789762731</v>
@@ -7533,16 +7509,16 @@
         <v>46212.77746881945</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="H102" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="H102" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="5">
@@ -7558,13 +7534,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="Q102" s="6"/>
       <c r="R102" s="6"/>
@@ -7574,7 +7550,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B103" s="9">
         <v>46146.78790538195</v>
@@ -7584,16 +7560,16 @@
         <v>46212.77748577546</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H103" s="10" t="s">
         <v>226</v>
-      </c>
-      <c r="H103" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="9">
@@ -7609,13 +7585,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="O103" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="Q103" s="10"/>
       <c r="R103" s="10"/>
@@ -7625,7 +7601,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B104" s="5">
         <v>46146.787928171296</v>
@@ -7635,16 +7611,16 @@
         <v>46146.94327527778</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="H104" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="H104" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="5">
@@ -7660,13 +7636,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="Q104" s="5">
         <v>46239</v>
@@ -7675,18 +7651,18 @@
         <v>46239</v>
       </c>
       <c r="S104" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T104" s="6">
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B105" s="9">
         <v>46146.787934409724</v>
@@ -7696,16 +7672,16 @@
         <v>46212.77751017361</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H105" s="10" t="s">
         <v>226</v>
-      </c>
-      <c r="H105" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="I105" s="10"/>
       <c r="J105" s="9">
@@ -7721,13 +7697,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="O105" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="Q105" s="10"/>
       <c r="R105" s="10"/>
@@ -7737,7 +7713,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B106" s="5">
         <v>46146.787939131944</v>
@@ -7747,16 +7723,16 @@
         <v>46212.777535706016</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G106" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="H106" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="H106" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="I106" s="6"/>
       <c r="J106" s="5">
@@ -7772,13 +7748,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7788,7 +7764,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B107" s="9">
         <v>46146.787957974535</v>
@@ -7798,7 +7774,7 @@
         <v>46146.94056351852</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>25</v>
@@ -7822,7 +7798,7 @@
         <v>26</v>
       </c>
       <c r="O107" s="10" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="P107" s="10" t="s">
         <v>26</v>
@@ -7835,7 +7811,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B108" s="5">
         <v>46146.78796153935</v>
@@ -7845,16 +7821,16 @@
         <v>46146.94352958333</v>
       </c>
       <c r="E108" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="F108" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G108" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="F108" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G108" s="6" t="s">
+      <c r="H108" s="6" t="s">
         <v>338</v>
-      </c>
-      <c r="H108" s="6" t="s">
-        <v>339</v>
       </c>
       <c r="I108" s="5">
         <v>46240</v>
@@ -7872,13 +7848,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="Q108" s="5">
         <v>46240</v>
@@ -7887,18 +7863,18 @@
         <v>46248</v>
       </c>
       <c r="S108" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T108" s="6">
         <v>0</v>
       </c>
       <c r="U108" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B109" s="9">
         <v>46146.78796724537</v>
@@ -7908,16 +7884,16 @@
         <v>46196.86770128472</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G109" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H109" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="H109" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="I109" s="9">
         <v>46240</v>
@@ -7935,13 +7911,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="O109" s="10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P109" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="Q109" s="9">
         <v>46240</v>
@@ -7950,13 +7926,13 @@
         <v>46248</v>
       </c>
       <c r="S109" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T109" s="10">
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-13 14:44 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -685,7 +685,7 @@
     <t>victor.munoz@zitron.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Bodega:,Control de calidad corte laser </t>
+    <t xml:space="preserve">Bodega:,Control de calidad corte laser ,Control de calidad corte laser </t>
   </si>
   <si>
     <t>1214511245146577</t>
@@ -4752,7 +4752,7 @@
         <v>46212.77629162037</v>
       </c>
       <c r="D54" s="5">
-        <v>46212.77630914352</v>
+        <v>46216.60292806713</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-22 15:05 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -748,7 +748,7 @@
     <t>nicolas.mol@zitron.com</t>
   </si>
   <si>
-    <t>OT 4309 - ZVN 1-9-75/2,OT2 4307 ZVN 1-9-86/2 ,OT 4375 - ZVN 1-9-86/2 + TOB + REJ + TIPO A,OT 4376 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,OT 4377-ZVN 1-9-86/2 + TOB + REJ + TPA</t>
+    <t xml:space="preserve">OT 4309 - ZVN 1-9-75/2,OT2 4307 ZVN 1-9-86/2 ,OT 4375 - ZVN 1-9-86/2 + TOB + REJ + TIPO A,OT 4376 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,OT 4377-ZVN 1-9-86/2 + TOB + REJ + TPA,OT4378-ZVN 1-9-63/2 + TOB + REJ + 2FAR + TIPO A </t>
   </si>
   <si>
     <t>1214508463084766</t>
@@ -5187,7 +5187,7 @@
         <v>46198.893461747684</v>
       </c>
       <c r="D61" s="9">
-        <v>46225.00960046296</v>
+        <v>46225.58945297454</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>222</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-03 15:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -748,7 +748,7 @@
     <t>nicolas.mol@zitron.com</t>
   </si>
   <si>
-    <t>OT 4309 - ZVN 1-9-75/2,OT2 4307 ZVN 1-9-86/2 ,OT 4375 - ZVN 1-9-86/2 + TOB + REJ + TIPO A,OT 4376 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,OT 4377-ZVN 1-9-86/2 + TOB + REJ + TPA,OT4378-ZVN 1-9-63/2 + TOB + REJ + 2FAR + TIPO A ,OT 4381 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,ot  4382 -ZVN 1-9-86/2 + TOB+ REJ + TIPO A ,ot  4385 -VENTILADORES 45KCFMx4"CA - ZVN 1-12-37/4</t>
+    <t>OT 4309 - ZVN 1-9-75/2,OT2 4307 ZVN 1-9-86/2 ,OT 4375 - ZVN 1-9-86/2 + TOB + REJ + TIPO A,OT 4376 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,OT 4377-ZVN 1-9-86/2 + TOB + REJ + TPA,OT4378-ZVN 1-9-63/2 + TOB + REJ + 2FAR + TIPO A ,OT 4381 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,ot  4382 -ZVN 1-9-86/2 + TOB+ REJ + TIPO A ,ot  4385 -VENTILADORES 45KCFMx4"CA - ZVN 1-12-37/4,ot  4385 -VENTILADORES 45KCFMx4"CA - ZVN 1-12-37/4,OT 4394 -ZVN 1-9-86/2 + TOB + REJ</t>
   </si>
   <si>
     <t>1214508463084766</t>
@@ -5190,7 +5190,7 @@
         <v>46198.893461747684</v>
       </c>
       <c r="D61" s="9">
-        <v>46233.64826086805</v>
+        <v>46237.57049788194</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>222</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-26 23:06 UTC
</commit_message>
<xml_diff>
--- a/data/50001543 - ZITRON COLOMBIA EGM.xlsx
+++ b/data/50001543 - ZITRON COLOMBIA EGM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1307" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="339">
   <si>
     <t>50001543 - ZITRON COLOMBIA EGM</t>
   </si>
@@ -6013,9 +6013,11 @@
       <c r="B75" s="9">
         <v>46146.78750452546</v>
       </c>
-      <c r="C75" s="10"/>
+      <c r="C75" s="9">
+        <v>46260.84442424768</v>
+      </c>
       <c r="D75" s="9">
-        <v>46260.83940523148</v>
+        <v>46260.84444311343</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>260</v>
@@ -6050,9 +6052,11 @@
       <c r="Q75" s="10"/>
       <c r="R75" s="10"/>
       <c r="S75" s="10"/>
-      <c r="T75" s="10"/>
-      <c r="U75" s="12" t="s">
-        <v>207</v>
+      <c r="T75" s="10">
+        <v>1</v>
+      </c>
+      <c r="U75" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -7086,7 +7090,7 @@
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46260.83942512731</v>
+        <v>46260.84455974537</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>302</v>
@@ -7122,7 +7126,9 @@
       <c r="R94" s="6"/>
       <c r="S94" s="6"/>
       <c r="T94" s="6"/>
-      <c r="U94" s="6"/>
+      <c r="U94" s="12" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
@@ -7131,9 +7137,11 @@
       <c r="B95" s="9">
         <v>46146.78778912037</v>
       </c>
-      <c r="C95" s="10"/>
+      <c r="C95" s="9">
+        <v>46260.84449711806</v>
+      </c>
       <c r="D95" s="9">
-        <v>46260.83939849537</v>
+        <v>46260.84451005787</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>305</v>
@@ -7179,10 +7187,10 @@
         <v>33</v>
       </c>
       <c r="T95" s="10">
-        <v>0</v>
-      </c>
-      <c r="U95" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U95" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
@@ -7192,9 +7200,11 @@
       <c r="B96" s="5">
         <v>46146.78779429398</v>
       </c>
-      <c r="C96" s="6"/>
+      <c r="C96" s="5">
+        <v>46260.84448118055</v>
+      </c>
       <c r="D96" s="5">
-        <v>46260.839191493054</v>
+        <v>46260.844482615736</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>191</v>
@@ -7243,9 +7253,11 @@
       <c r="B97" s="9">
         <v>46146.787798414356</v>
       </c>
-      <c r="C97" s="10"/>
+      <c r="C97" s="9">
+        <v>46260.844485787035</v>
+      </c>
       <c r="D97" s="9">
-        <v>46260.839378668985</v>
+        <v>46260.84448701389</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>191</v>
@@ -7359,7 +7371,7 @@
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46237.16882690972</v>
+        <v>46260.844491724536</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>191</v>
@@ -7410,7 +7422,7 @@
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46237.16882849537</v>
+        <v>46260.84449135417</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>191</v>
@@ -7463,7 +7475,7 @@
         <v>46260.83941804398</v>
       </c>
       <c r="D101" s="9">
-        <v>46260.83943501157</v>
+        <v>46260.83958581019</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>320</v>
@@ -7511,8 +7523,8 @@
       <c r="T101" s="10">
         <v>1</v>
       </c>
-      <c r="U101" s="7" t="s">
-        <v>27</v>
+      <c r="U101" s="12" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
@@ -7522,9 +7534,11 @@
       <c r="B102" s="5">
         <v>46146.78789762731</v>
       </c>
-      <c r="C102" s="6"/>
+      <c r="C102" s="5">
+        <v>46260.83956966436</v>
+      </c>
       <c r="D102" s="5">
-        <v>46238.1680128588</v>
+        <v>46260.839570972224</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>191</v>
@@ -7573,9 +7587,11 @@
       <c r="B103" s="9">
         <v>46146.78790538195</v>
       </c>
-      <c r="C103" s="10"/>
+      <c r="C103" s="9">
+        <v>46260.83951644676</v>
+      </c>
       <c r="D103" s="9">
-        <v>46238.1680141088</v>
+        <v>46260.83951788195</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>191</v>
@@ -7624,9 +7640,11 @@
       <c r="B104" s="5">
         <v>46146.787928171296</v>
       </c>
-      <c r="C104" s="6"/>
+      <c r="C104" s="5">
+        <v>46260.844537638885</v>
+      </c>
       <c r="D104" s="5">
-        <v>46260.57514836805</v>
+        <v>46260.8445503588</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>326</v>
@@ -7672,10 +7690,10 @@
         <v>33</v>
       </c>
       <c r="T104" s="6">
-        <v>0</v>
-      </c>
-      <c r="U104" s="7" t="s">
-        <v>27</v>
+        <v>1</v>
+      </c>
+      <c r="U104" s="12" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7685,9 +7703,11 @@
       <c r="B105" s="9">
         <v>46146.787934409724</v>
       </c>
-      <c r="C105" s="10"/>
+      <c r="C105" s="9">
+        <v>46260.84451734954</v>
+      </c>
       <c r="D105" s="9">
-        <v>46239.167930972224</v>
+        <v>46260.84451940972</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>191</v>
@@ -7736,9 +7756,11 @@
       <c r="B106" s="5">
         <v>46146.787939131944</v>
       </c>
-      <c r="C106" s="6"/>
+      <c r="C106" s="5">
+        <v>46260.84452320602</v>
+      </c>
       <c r="D106" s="5">
-        <v>46239.167932233795</v>
+        <v>46260.84452525463</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>191</v>
@@ -7836,7 +7858,7 @@
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46249.181991273144</v>
+        <v>46260.84456067129</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>334</v>
@@ -7886,8 +7908,8 @@
       <c r="T108" s="6">
         <v>0</v>
       </c>
-      <c r="U108" s="11" t="s">
-        <v>102</v>
+      <c r="U108" s="12" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
@@ -7899,7 +7921,7 @@
       </c>
       <c r="C109" s="10"/>
       <c r="D109" s="9">
-        <v>46249.181991273144</v>
+        <v>46260.8445634838</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>338</v>
@@ -7949,8 +7971,8 @@
       <c r="T109" s="10">
         <v>0</v>
       </c>
-      <c r="U109" s="11" t="s">
-        <v>102</v>
+      <c r="U109" s="12" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>